<commit_message>
Alterações finais no gerador de relatórios
</commit_message>
<xml_diff>
--- a/src/planilha_fiscalizacao.xlsx
+++ b/src/planilha_fiscalizacao.xlsx
@@ -3,13 +3,11 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fiscalizações" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Não-conformidades " sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Observações Importantes" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Recomendações" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="0" fullCalcOnLoad="1"/>
@@ -19,13 +17,18 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="3">
+  <fonts count="4">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <sz val="11"/>
     </font>
     <font>
       <name val="Calibri"/>
@@ -77,12 +80,18 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top"/>
     </xf>
   </cellXfs>
@@ -450,7 +459,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K13"/>
+  <dimension ref="A1:K16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -467,57 +476,57 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="2" t="inlineStr">
+      <c r="A1" s="4" t="inlineStr">
         <is>
           <t>ID da Fiscalização</t>
         </is>
       </c>
-      <c r="B1" s="2" t="inlineStr">
+      <c r="B1" s="4" t="inlineStr">
         <is>
           <t>Data</t>
         </is>
       </c>
-      <c r="C1" s="2" t="inlineStr">
+      <c r="C1" s="4" t="inlineStr">
         <is>
           <t>Hora</t>
         </is>
       </c>
-      <c r="D1" s="2" t="inlineStr">
+      <c r="D1" s="4" t="inlineStr">
         <is>
           <t>Cidade</t>
         </is>
       </c>
-      <c r="E1" s="2" t="inlineStr">
+      <c r="E1" s="4" t="inlineStr">
         <is>
           <t>Local</t>
         </is>
       </c>
-      <c r="F1" s="2" t="inlineStr">
+      <c r="F1" s="4" t="inlineStr">
         <is>
           <t>Pessoal Responsável</t>
         </is>
       </c>
-      <c r="G1" s="2" t="inlineStr">
+      <c r="G1" s="4" t="inlineStr">
         <is>
           <t>Coordenador</t>
         </is>
       </c>
-      <c r="H1" s="2" t="inlineStr">
+      <c r="H1" s="4" t="inlineStr">
         <is>
           <t>Contrato</t>
         </is>
       </c>
-      <c r="I1" s="2" t="inlineStr">
+      <c r="I1" s="4" t="inlineStr">
         <is>
           <t>Período</t>
         </is>
       </c>
-      <c r="J1" s="2" t="inlineStr">
+      <c r="J1" s="4" t="inlineStr">
         <is>
           <t>Assinatura</t>
         </is>
       </c>
-      <c r="K1" s="2" t="inlineStr">
+      <c r="K1" s="4" t="inlineStr">
         <is>
           <t>Relatório Gerado</t>
         </is>
@@ -688,22 +697,17 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>11/06/2025</t>
+          <t>11/03/2025</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>10:00:09</t>
+          <t>10:50:00</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Joao Recife Pessoas</t>
-        </is>
-      </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>Terminal Rodoviário do Recife - TIP</t>
+          <t>Recife</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
@@ -718,12 +722,12 @@
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>Nº 1.041.080/17</t>
+          <t>Nº 1.041.080/08</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>26/04/2025 a 01/05/2034</t>
+          <t>22/09/2025 a 26/09/2025</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
@@ -1156,6 +1160,165 @@
         </is>
       </c>
       <c r="K13" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="n">
+        <v>13</v>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>12/06/2026</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>10:00:18</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>Recife</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>Terminal Rodoviário do Recife - TIP</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>Débora Marcolino e Enildo Manoel</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>Maria Ângela Albuquerque de Freitas</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>Nº 1.041.080/09</t>
+        </is>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>26/04/2025 a 01/05/2042</t>
+        </is>
+      </c>
+      <c r="J14" t="inlineStr">
+        <is>
+          <t>Débora Marcolino;Enildo Manoel</t>
+        </is>
+      </c>
+      <c r="K14" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="n">
+        <v>15</v>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>12/06/2027</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>10:00:19</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>Recife</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>Terminal Rodoviário do Recife - TIP</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>Débora Marcolino e Enildo Manoel</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>Maria Ângela Albuquerque de Freitas</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>Nº 1.041.080/10</t>
+        </is>
+      </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>26/04/2025 a 01/05/2043</t>
+        </is>
+      </c>
+      <c r="J15" t="inlineStr">
+        <is>
+          <t>Débora Marcolino;Enildo Manoel</t>
+        </is>
+      </c>
+      <c r="K15" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="n">
+        <v>17</v>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>12/06/2027</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>10:00:19</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>Recife</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>Terminal Rodoviário do Recife - TIP</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>Débora Marcolino e Enildo Manoel</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>Maria Ângela Albuquerque de Freitas</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>Nº 1.041.080/10</t>
+        </is>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>26/04/2025 a 01/05/2043</t>
+        </is>
+      </c>
+      <c r="J16" t="inlineStr">
+        <is>
+          <t>Débora Marcolino;Enildo Manoel</t>
+        </is>
+      </c>
+      <c r="K16" t="b">
         <v>1</v>
       </c>
     </row>
@@ -1170,36 +1333,74 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F71"/>
+  <dimension ref="A1:K95"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="20" customWidth="1" min="1" max="1"/>
+    <col width="33" customWidth="1" min="2" max="2"/>
+    <col width="61" customWidth="1" min="3" max="3"/>
+    <col width="526" customWidth="1" min="4" max="4"/>
+    <col width="20" customWidth="1" min="5" max="5"/>
+    <col width="13" customWidth="1" min="6" max="6"/>
+    <col width="17" customWidth="1" min="7" max="7"/>
+    <col width="48" customWidth="1" min="8" max="8"/>
+    <col width="25" customWidth="1" min="9" max="9"/>
+    <col width="25" customWidth="1" min="10" max="10"/>
+    <col width="533" customWidth="1" min="11" max="11"/>
+  </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="2" t="inlineStr">
+      <c r="A1" s="4" t="inlineStr">
         <is>
           <t>ID da Fiscalização</t>
         </is>
       </c>
-      <c r="B1" s="2" t="inlineStr">
-        <is>
-          <t>Nº</t>
-        </is>
-      </c>
-      <c r="C1" s="2" t="inlineStr">
+      <c r="B1" s="4" t="inlineStr">
         <is>
           <t>Terminal</t>
         </is>
       </c>
-      <c r="D1" s="2" t="inlineStr">
+      <c r="C1" s="4" t="inlineStr">
+        <is>
+          <t>ID da não conformidade</t>
+        </is>
+      </c>
+      <c r="D1" s="4" t="inlineStr">
         <is>
           <t>Não Conformidade</t>
         </is>
       </c>
-      <c r="E1" s="2" t="inlineStr">
-        <is>
-          <t>Foto</t>
-        </is>
-      </c>
-      <c r="F1" s="2" t="inlineStr">
+      <c r="E1" s="4" t="inlineStr">
+        <is>
+          <t>Informação SOCICAM</t>
+        </is>
+      </c>
+      <c r="F1" s="4" t="inlineStr">
+        <is>
+          <t>Constatação</t>
+        </is>
+      </c>
+      <c r="G1" s="4" t="inlineStr">
+        <is>
+          <t>Análise da Arpe</t>
+        </is>
+      </c>
+      <c r="H1" s="4" t="inlineStr">
+        <is>
+          <t>Informação SOCICAM carta</t>
+        </is>
+      </c>
+      <c r="I1" s="4" t="inlineStr">
+        <is>
+          <t>Vistoria da Arpe</t>
+        </is>
+      </c>
+      <c r="J1" s="4" t="inlineStr">
+        <is>
+          <t>Situação</t>
+        </is>
+      </c>
+      <c r="K1" s="4" t="inlineStr">
         <is>
           <t>Legenda da Foto</t>
         </is>
@@ -1209,10 +1410,7 @@
       <c r="A2" t="n">
         <v>1</v>
       </c>
-      <c r="B2" t="n">
-        <v>1.1</v>
-      </c>
-      <c r="C2" t="inlineStr">
+      <c r="B2" t="inlineStr">
         <is>
           <t>Terminal do Recife (TIP)</t>
         </is>
@@ -1222,12 +1420,7 @@
           <t>CIMENTO NÃO POSICIONADO NA SACADA</t>
         </is>
       </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>foto01.jpg</t>
-        </is>
-      </c>
-      <c r="F2" t="inlineStr">
+      <c r="K2" t="inlineStr">
         <is>
           <t>Infiltração em coluna de sustentação do Terminal do recife</t>
         </is>
@@ -1237,10 +1430,7 @@
       <c r="A3" t="n">
         <v>1</v>
       </c>
-      <c r="B3" t="n">
-        <v>1.2</v>
-      </c>
-      <c r="C3" t="inlineStr">
+      <c r="B3" t="inlineStr">
         <is>
           <t>Terminal do Recife (TIP)</t>
         </is>
@@ -1250,7 +1440,7 @@
           <t>CIMENTO NÃO POSICIONADO NA SACADA</t>
         </is>
       </c>
-      <c r="F3" t="inlineStr">
+      <c r="K3" t="inlineStr">
         <is>
           <t>Infiltração em coluna de sustentação do Terminal do recife</t>
         </is>
@@ -1260,10 +1450,7 @@
       <c r="A4" t="n">
         <v>1</v>
       </c>
-      <c r="B4" t="n">
-        <v>1.3</v>
-      </c>
-      <c r="C4" t="inlineStr">
+      <c r="B4" t="inlineStr">
         <is>
           <t>Terminal do Recife (TIP)</t>
         </is>
@@ -1273,12 +1460,7 @@
           <t>CIMENTO NÃO POSICIONADO NA SACADA</t>
         </is>
       </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>foto01.jpg</t>
-        </is>
-      </c>
-      <c r="F4" t="inlineStr">
+      <c r="K4" t="inlineStr">
         <is>
           <t>Infiltração em coluna de sustentação do Terminal do recife</t>
         </is>
@@ -1288,10 +1470,7 @@
       <c r="A5" t="n">
         <v>1</v>
       </c>
-      <c r="B5" t="n">
-        <v>1.4</v>
-      </c>
-      <c r="C5" t="inlineStr">
+      <c r="B5" t="inlineStr">
         <is>
           <t>Terminal de Petrolina</t>
         </is>
@@ -1301,12 +1480,7 @@
           <t>CIMENTO NÃO POSICIONADO NA SACADA</t>
         </is>
       </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>foto01.jpg</t>
-        </is>
-      </c>
-      <c r="F5" t="inlineStr">
+      <c r="K5" t="inlineStr">
         <is>
           <t>Infiltração em coluna de sustentação do Terminal do recife</t>
         </is>
@@ -1316,10 +1490,7 @@
       <c r="A6" t="n">
         <v>1</v>
       </c>
-      <c r="B6" t="n">
-        <v>1.5</v>
-      </c>
-      <c r="C6" t="inlineStr">
+      <c r="B6" t="inlineStr">
         <is>
           <t>Terminal de Caruaru</t>
         </is>
@@ -1329,12 +1500,7 @@
           <t>CIMENTO NÃO POSICIONADO NA SACADA</t>
         </is>
       </c>
-      <c r="E6" t="inlineStr">
-        <is>
-          <t>foto01.jpg</t>
-        </is>
-      </c>
-      <c r="F6" t="inlineStr">
+      <c r="K6" t="inlineStr">
         <is>
           <t>Infiltração em coluna de sustentação do Terminal do recife</t>
         </is>
@@ -1344,10 +1510,7 @@
       <c r="A7" t="n">
         <v>1</v>
       </c>
-      <c r="B7" t="n">
-        <v>1.6</v>
-      </c>
-      <c r="C7" t="inlineStr">
+      <c r="B7" t="inlineStr">
         <is>
           <t>Terminal de Garanhuns</t>
         </is>
@@ -1357,12 +1520,7 @@
           <t>CIMENTO NÃO POSICIONADO NA SACADA</t>
         </is>
       </c>
-      <c r="E7" t="inlineStr">
-        <is>
-          <t>foto01.jpg</t>
-        </is>
-      </c>
-      <c r="F7" t="inlineStr">
+      <c r="K7" t="inlineStr">
         <is>
           <t>Infiltração em coluna de sustentação do Terminal do recife</t>
         </is>
@@ -1372,10 +1530,7 @@
       <c r="A8" t="n">
         <v>1</v>
       </c>
-      <c r="B8" t="n">
-        <v>1.7</v>
-      </c>
-      <c r="C8" t="inlineStr">
+      <c r="B8" t="inlineStr">
         <is>
           <t>Terminal de Arcoverde</t>
         </is>
@@ -1385,12 +1540,7 @@
           <t>CIMENTO NÃO POSICIONADO NA SACADA</t>
         </is>
       </c>
-      <c r="E8" t="inlineStr">
-        <is>
-          <t>foto01.jpg</t>
-        </is>
-      </c>
-      <c r="F8" t="inlineStr">
+      <c r="K8" t="inlineStr">
         <is>
           <t>Infiltração em coluna de sustentação do Terminal do recife</t>
         </is>
@@ -1400,10 +1550,7 @@
       <c r="A9" t="n">
         <v>1</v>
       </c>
-      <c r="B9" t="n">
-        <v>1.8</v>
-      </c>
-      <c r="C9" t="inlineStr">
+      <c r="B9" t="inlineStr">
         <is>
           <t>Terminal de Arcoverde</t>
         </is>
@@ -1413,12 +1560,7 @@
           <t>CIMENTO NÃO POSICIONADO NA SACADA</t>
         </is>
       </c>
-      <c r="E9" t="inlineStr">
-        <is>
-          <t>foto01.jpg</t>
-        </is>
-      </c>
-      <c r="F9" t="inlineStr">
+      <c r="K9" t="inlineStr">
         <is>
           <t>Infiltração em coluna de sustentação do Terminal do recife</t>
         </is>
@@ -1428,10 +1570,7 @@
       <c r="A10" t="n">
         <v>1</v>
       </c>
-      <c r="B10" t="n">
-        <v>1.9</v>
-      </c>
-      <c r="C10" t="inlineStr">
+      <c r="B10" t="inlineStr">
         <is>
           <t>Terminal de Arcoverde</t>
         </is>
@@ -1441,12 +1580,7 @@
           <t>CIMENTO NÃO POSICIONADO NA SACADA</t>
         </is>
       </c>
-      <c r="E10" t="inlineStr">
-        <is>
-          <t>foto01.jpg</t>
-        </is>
-      </c>
-      <c r="F10" t="inlineStr">
+      <c r="K10" t="inlineStr">
         <is>
           <t>Infiltração em coluna de sustentação do Terminal do recife</t>
         </is>
@@ -1456,10 +1590,7 @@
       <c r="A11" t="n">
         <v>1</v>
       </c>
-      <c r="B11" t="n">
-        <v>2</v>
-      </c>
-      <c r="C11" t="inlineStr">
+      <c r="B11" t="inlineStr">
         <is>
           <t>Terminal de Arcoverde</t>
         </is>
@@ -1469,12 +1600,7 @@
           <t>CIMENTO NÃO POSICIONADO NA SACADA</t>
         </is>
       </c>
-      <c r="E11" t="inlineStr">
-        <is>
-          <t>foto01.jpg</t>
-        </is>
-      </c>
-      <c r="F11" t="inlineStr">
+      <c r="K11" t="inlineStr">
         <is>
           <t>Infiltração em coluna de sustentação do Terminal do recife</t>
         </is>
@@ -1484,10 +1610,7 @@
       <c r="A12" t="n">
         <v>7</v>
       </c>
-      <c r="B12" t="n">
-        <v>1.1</v>
-      </c>
-      <c r="C12" t="inlineStr">
+      <c r="B12" t="inlineStr">
         <is>
           <t>Terminal de Caruaru</t>
         </is>
@@ -1497,12 +1620,7 @@
           <t>CIMENTO NÃO POSICIONADO NA SACADA</t>
         </is>
       </c>
-      <c r="E12" t="inlineStr">
-        <is>
-          <t>foto01.jpg</t>
-        </is>
-      </c>
-      <c r="F12" t="inlineStr">
+      <c r="K12" t="inlineStr">
         <is>
           <t>Infiltração em coluna de sustentação do Terminal do recife</t>
         </is>
@@ -1512,10 +1630,7 @@
       <c r="A13" t="n">
         <v>7</v>
       </c>
-      <c r="B13" t="n">
-        <v>1.1</v>
-      </c>
-      <c r="C13" t="inlineStr">
+      <c r="B13" t="inlineStr">
         <is>
           <t>Terminal de Garanhuns</t>
         </is>
@@ -1525,12 +1640,7 @@
           <t>CIMENTO NÃO POSICIONADO NA SACADA</t>
         </is>
       </c>
-      <c r="E13" t="inlineStr">
-        <is>
-          <t>foto01.jpg</t>
-        </is>
-      </c>
-      <c r="F13" t="inlineStr">
+      <c r="K13" t="inlineStr">
         <is>
           <t>Infiltração em coluna de sustentação do Terminal do recife</t>
         </is>
@@ -1540,10 +1650,7 @@
       <c r="A14" t="n">
         <v>7</v>
       </c>
-      <c r="B14" t="n">
-        <v>1.1</v>
-      </c>
-      <c r="C14" t="inlineStr">
+      <c r="B14" t="inlineStr">
         <is>
           <t>Terminal de Arcoverde</t>
         </is>
@@ -1553,12 +1660,7 @@
           <t>CIMENTO NÃO POSICIONADO NA SACADA</t>
         </is>
       </c>
-      <c r="E14" t="inlineStr">
-        <is>
-          <t>foto01.jpg</t>
-        </is>
-      </c>
-      <c r="F14" t="inlineStr">
+      <c r="K14" t="inlineStr">
         <is>
           <t>Infiltração em coluna de sustentação do Terminal do recife</t>
         </is>
@@ -1568,10 +1670,7 @@
       <c r="A15" t="n">
         <v>7</v>
       </c>
-      <c r="B15" t="n">
-        <v>1.1</v>
-      </c>
-      <c r="C15" t="inlineStr">
+      <c r="B15" t="inlineStr">
         <is>
           <t>Terminal de Arcoverde</t>
         </is>
@@ -1581,12 +1680,7 @@
           <t>CIMENTO NÃO POSICIONADO NA SACADA</t>
         </is>
       </c>
-      <c r="E15" t="inlineStr">
-        <is>
-          <t>foto01.jpg</t>
-        </is>
-      </c>
-      <c r="F15" t="inlineStr">
+      <c r="K15" t="inlineStr">
         <is>
           <t>Infiltração em coluna de sustentação do Terminal do recife</t>
         </is>
@@ -1596,10 +1690,7 @@
       <c r="A16" t="n">
         <v>7</v>
       </c>
-      <c r="B16" t="n">
-        <v>1.1</v>
-      </c>
-      <c r="C16" t="inlineStr">
+      <c r="B16" t="inlineStr">
         <is>
           <t>Terminal de Garanhuns</t>
         </is>
@@ -1609,12 +1700,7 @@
           <t>CIMENTO NÃO POSICIONADO NA SACADA</t>
         </is>
       </c>
-      <c r="E16" t="inlineStr">
-        <is>
-          <t>foto01.jpg</t>
-        </is>
-      </c>
-      <c r="F16" t="inlineStr">
+      <c r="K16" t="inlineStr">
         <is>
           <t>Infiltração em coluna de sustentação do Terminal do recife</t>
         </is>
@@ -1624,10 +1710,7 @@
       <c r="A17" t="n">
         <v>7</v>
       </c>
-      <c r="B17" t="n">
-        <v>1.1</v>
-      </c>
-      <c r="C17" t="inlineStr">
+      <c r="B17" t="inlineStr">
         <is>
           <t>Terminal de Garanhuns</t>
         </is>
@@ -1637,12 +1720,7 @@
           <t>CIMENTO NÃO POSICIONADO NA SACADA</t>
         </is>
       </c>
-      <c r="E17" t="inlineStr">
-        <is>
-          <t>foto01.jpg</t>
-        </is>
-      </c>
-      <c r="F17" t="inlineStr">
+      <c r="K17" t="inlineStr">
         <is>
           <t>Infiltração em coluna de sustentação do Terminal do recife</t>
         </is>
@@ -1652,10 +1730,7 @@
       <c r="A18" t="n">
         <v>7</v>
       </c>
-      <c r="B18" t="n">
-        <v>1.1</v>
-      </c>
-      <c r="C18" t="inlineStr">
+      <c r="B18" t="inlineStr">
         <is>
           <t>Terminal de Arcoverde</t>
         </is>
@@ -1665,7 +1740,7 @@
           <t>CIMENTO NÃO POSICIONADO NA SACADA</t>
         </is>
       </c>
-      <c r="F18" t="inlineStr">
+      <c r="K18" t="inlineStr">
         <is>
           <t>Infiltração em coluna de sustentação do Terminal do recife</t>
         </is>
@@ -1675,10 +1750,7 @@
       <c r="A19" t="n">
         <v>9</v>
       </c>
-      <c r="B19" t="n">
-        <v>1.1</v>
-      </c>
-      <c r="C19" t="inlineStr">
+      <c r="B19" t="inlineStr">
         <is>
           <t>Terminal de Arcoverde</t>
         </is>
@@ -1688,12 +1760,7 @@
           <t>CIMENTO NÃO POSICIONADO NA SACADA</t>
         </is>
       </c>
-      <c r="E19" t="inlineStr">
-        <is>
-          <t>foto01.jpg</t>
-        </is>
-      </c>
-      <c r="F19" t="inlineStr">
+      <c r="K19" t="inlineStr">
         <is>
           <t>Infiltração em coluna de sustentação do Terminal do recife</t>
         </is>
@@ -1703,10 +1770,7 @@
       <c r="A20" t="n">
         <v>9</v>
       </c>
-      <c r="B20" t="n">
-        <v>1.1</v>
-      </c>
-      <c r="C20" t="inlineStr">
+      <c r="B20" t="inlineStr">
         <is>
           <t>Terminal de Arcoverde</t>
         </is>
@@ -1716,12 +1780,7 @@
           <t>CIMENTO NÃO POSICIONADO NA SACADA</t>
         </is>
       </c>
-      <c r="E20" t="inlineStr">
-        <is>
-          <t>foto01.jpg</t>
-        </is>
-      </c>
-      <c r="F20" t="inlineStr">
+      <c r="K20" t="inlineStr">
         <is>
           <t>Infiltração em coluna de sustentação do Terminal do recife</t>
         </is>
@@ -1731,10 +1790,7 @@
       <c r="A21" t="n">
         <v>9</v>
       </c>
-      <c r="B21" t="n">
-        <v>1.1</v>
-      </c>
-      <c r="C21" t="inlineStr">
+      <c r="B21" t="inlineStr">
         <is>
           <t>Terminal de Arcoverde</t>
         </is>
@@ -1744,12 +1800,7 @@
           <t>CIMENTO NÃO POSICIONADO NA SACADA</t>
         </is>
       </c>
-      <c r="E21" t="inlineStr">
-        <is>
-          <t>foto01.jpg</t>
-        </is>
-      </c>
-      <c r="F21" t="inlineStr">
+      <c r="K21" t="inlineStr">
         <is>
           <t>Infiltração em coluna de sustentação do Terminal do recife</t>
         </is>
@@ -1759,10 +1810,7 @@
       <c r="A22" t="n">
         <v>9</v>
       </c>
-      <c r="B22" t="n">
-        <v>1.1</v>
-      </c>
-      <c r="C22" t="inlineStr">
+      <c r="B22" t="inlineStr">
         <is>
           <t>Terminal de Arcoverde</t>
         </is>
@@ -1772,12 +1820,7 @@
           <t>CIMENTO NÃO POSICIONADO NA SACADA</t>
         </is>
       </c>
-      <c r="E22" t="inlineStr">
-        <is>
-          <t>foto01.jpg</t>
-        </is>
-      </c>
-      <c r="F22" t="inlineStr">
+      <c r="K22" t="inlineStr">
         <is>
           <t>Infiltração em coluna de sustentação do Terminal do recife</t>
         </is>
@@ -1787,10 +1830,7 @@
       <c r="A23" t="n">
         <v>9</v>
       </c>
-      <c r="B23" t="n">
-        <v>1.1</v>
-      </c>
-      <c r="C23" t="inlineStr">
+      <c r="B23" t="inlineStr">
         <is>
           <t>Terminal de Arcoverde</t>
         </is>
@@ -1800,12 +1840,7 @@
           <t>CIMENTO NÃO POSICIONADO NA SACADA</t>
         </is>
       </c>
-      <c r="E23" t="inlineStr">
-        <is>
-          <t>foto01.jpg</t>
-        </is>
-      </c>
-      <c r="F23" t="inlineStr">
+      <c r="K23" t="inlineStr">
         <is>
           <t>Infiltração em coluna de sustentação do Terminal do recife</t>
         </is>
@@ -1815,10 +1850,7 @@
       <c r="A24" t="n">
         <v>9</v>
       </c>
-      <c r="B24" t="n">
-        <v>1.1</v>
-      </c>
-      <c r="C24" t="inlineStr">
+      <c r="B24" t="inlineStr">
         <is>
           <t>Terminal de Arcoverde</t>
         </is>
@@ -1828,12 +1860,7 @@
           <t>CIMENTO NÃO POSICIONADO NA SACADA</t>
         </is>
       </c>
-      <c r="E24" t="inlineStr">
-        <is>
-          <t>foto01.jpg</t>
-        </is>
-      </c>
-      <c r="F24" t="inlineStr">
+      <c r="K24" t="inlineStr">
         <is>
           <t>Infiltração em coluna de sustentação do Terminal do recife</t>
         </is>
@@ -1843,10 +1870,7 @@
       <c r="A25" t="n">
         <v>9</v>
       </c>
-      <c r="B25" t="n">
-        <v>1.1</v>
-      </c>
-      <c r="C25" t="inlineStr">
+      <c r="B25" t="inlineStr">
         <is>
           <t>Terminal de Arcoverde</t>
         </is>
@@ -1856,12 +1880,7 @@
           <t>CIMENTO NÃO POSICIONADO NA SACADA</t>
         </is>
       </c>
-      <c r="E25" t="inlineStr">
-        <is>
-          <t>foto01.jpg</t>
-        </is>
-      </c>
-      <c r="F25" t="inlineStr">
+      <c r="K25" t="inlineStr">
         <is>
           <t>Infiltração em coluna de sustentação do Terminal do recife</t>
         </is>
@@ -1871,10 +1890,7 @@
       <c r="A26" t="n">
         <v>9</v>
       </c>
-      <c r="B26" t="n">
-        <v>1.1</v>
-      </c>
-      <c r="C26" t="inlineStr">
+      <c r="B26" t="inlineStr">
         <is>
           <t>Terminal de Arcoverde</t>
         </is>
@@ -1884,12 +1900,7 @@
           <t>CIMENTO NÃO POSICIONADO NA SACADA</t>
         </is>
       </c>
-      <c r="E26" t="inlineStr">
-        <is>
-          <t>foto01.jpg</t>
-        </is>
-      </c>
-      <c r="F26" t="inlineStr">
+      <c r="K26" t="inlineStr">
         <is>
           <t>Infiltração em coluna de sustentação do Terminal do recife</t>
         </is>
@@ -1899,10 +1910,7 @@
       <c r="A27" t="n">
         <v>10</v>
       </c>
-      <c r="B27" t="n">
-        <v>1.1</v>
-      </c>
-      <c r="C27" t="inlineStr">
+      <c r="B27" t="inlineStr">
         <is>
           <t>Terminal de Arcoverde</t>
         </is>
@@ -1912,12 +1920,7 @@
           <t>CIMENTO NÃO POSICIONADO NA SACADA</t>
         </is>
       </c>
-      <c r="E27" t="inlineStr">
-        <is>
-          <t>foto01.jpg</t>
-        </is>
-      </c>
-      <c r="F27" t="inlineStr">
+      <c r="K27" t="inlineStr">
         <is>
           <t>Infiltração em coluna de sustentação do Terminal do recife</t>
         </is>
@@ -1927,10 +1930,7 @@
       <c r="A28" t="n">
         <v>10</v>
       </c>
-      <c r="B28" t="n">
-        <v>1.1</v>
-      </c>
-      <c r="C28" t="inlineStr">
+      <c r="B28" t="inlineStr">
         <is>
           <t>Terminal de Arcoverde</t>
         </is>
@@ -1940,7 +1940,7 @@
           <t>CIMENTO NÃO POSICIONADO NA SACADA</t>
         </is>
       </c>
-      <c r="F28" t="inlineStr">
+      <c r="K28" t="inlineStr">
         <is>
           <t>Infiltração em coluna de sustentação do Terminal do recife</t>
         </is>
@@ -1950,10 +1950,7 @@
       <c r="A29" t="n">
         <v>11</v>
       </c>
-      <c r="B29" t="n">
-        <v>1.1</v>
-      </c>
-      <c r="C29" t="inlineStr">
+      <c r="B29" t="inlineStr">
         <is>
           <t>Terminal do Recife (TIP)</t>
         </is>
@@ -1963,12 +1960,7 @@
           <t>Infiltração na coluna de sustentação da estrutura metálica da área de embarque e desembarque do Terminal do Recife (TIP), conforme evidenciado nas fotos 01 e 02, a seguir!!!!!!!</t>
         </is>
       </c>
-      <c r="E29" t="inlineStr">
-        <is>
-          <t>foto01.jpg;foto02.jpg</t>
-        </is>
-      </c>
-      <c r="F29" t="inlineStr">
+      <c r="K29" t="inlineStr">
         <is>
           <t>Infiltração em coluna de sustentação do Terminal do Recife em 20/03/2025.;Piso desgastado conforme evidência da foto 04.</t>
         </is>
@@ -1978,10 +1970,7 @@
       <c r="A30" t="n">
         <v>11</v>
       </c>
-      <c r="B30" t="n">
-        <v>1.1</v>
-      </c>
-      <c r="C30" t="inlineStr">
+      <c r="B30" t="inlineStr">
         <is>
           <t>Terminal do Recife (TIP)</t>
         </is>
@@ -1996,10 +1985,7 @@
       <c r="A31" t="n">
         <v>11</v>
       </c>
-      <c r="B31" t="n">
-        <v>1.2</v>
-      </c>
-      <c r="C31" t="inlineStr">
+      <c r="B31" t="inlineStr">
         <is>
           <t>Terminal do Recife (TIP)</t>
         </is>
@@ -2014,10 +2000,7 @@
       <c r="A32" t="n">
         <v>11</v>
       </c>
-      <c r="B32" t="n">
-        <v>1.3</v>
-      </c>
-      <c r="C32" t="inlineStr">
+      <c r="B32" t="inlineStr">
         <is>
           <t>Terminal do Recife (TIP)</t>
         </is>
@@ -2032,10 +2015,7 @@
       <c r="A33" t="n">
         <v>11</v>
       </c>
-      <c r="B33" t="n">
-        <v>1.4</v>
-      </c>
-      <c r="C33" t="inlineStr">
+      <c r="B33" t="inlineStr">
         <is>
           <t>Terminal do Recife (TIP)</t>
         </is>
@@ -2045,12 +2025,7 @@
           <t xml:space="preserve">Barra de apoio vertical oxidada, conforme foto 04, a seguir. </t>
         </is>
       </c>
-      <c r="E33" t="inlineStr">
-        <is>
-          <t>foto01.jpg;foto02.jpg</t>
-        </is>
-      </c>
-      <c r="F33" t="inlineStr">
+      <c r="K33" t="inlineStr">
         <is>
           <t>Espelho e barra em torno da pia oxidados no banehiro feminino PCD do Terminal de Recife, 20/03/2025;Infiltração em coluna de sustentação do Terminal do Recife em 20/03/2025</t>
         </is>
@@ -2060,10 +2035,7 @@
       <c r="A34" t="n">
         <v>11</v>
       </c>
-      <c r="B34" t="n">
-        <v>1.5</v>
-      </c>
-      <c r="C34" t="inlineStr">
+      <c r="B34" t="inlineStr">
         <is>
           <t>Terminal do Recife (TIP)</t>
         </is>
@@ -2073,12 +2045,7 @@
           <t>Piso desgastado na entrada do banheiro feminino do TIP em 20/03/2025;</t>
         </is>
       </c>
-      <c r="E34" t="inlineStr">
-        <is>
-          <t>foto01.jpg</t>
-        </is>
-      </c>
-      <c r="F34" t="inlineStr">
+      <c r="K34" t="inlineStr">
         <is>
           <t>Piso desgastado conforme evidência da foto 04.</t>
         </is>
@@ -2088,10 +2055,7 @@
       <c r="A35" t="n">
         <v>11</v>
       </c>
-      <c r="B35" t="n">
-        <v>1.6</v>
-      </c>
-      <c r="C35" t="inlineStr">
+      <c r="B35" t="inlineStr">
         <is>
           <t>Terminal de Caruaru (CAR)</t>
         </is>
@@ -2101,12 +2065,7 @@
           <t>Piso desgastado na entrada do banheiro feminino do TIP em 20/03/2025;</t>
         </is>
       </c>
-      <c r="E35" t="inlineStr">
-        <is>
-          <t>foto01.jpg</t>
-        </is>
-      </c>
-      <c r="F35" t="inlineStr">
+      <c r="K35" t="inlineStr">
         <is>
           <t>Piso desgastado conforme evidência da foto 04.</t>
         </is>
@@ -2116,10 +2075,7 @@
       <c r="A36" t="n">
         <v>11</v>
       </c>
-      <c r="B36" t="n">
-        <v>1.7</v>
-      </c>
-      <c r="C36" t="inlineStr">
+      <c r="B36" t="inlineStr">
         <is>
           <t>Terminal de Caruaru (CAR)</t>
         </is>
@@ -2129,12 +2085,7 @@
           <t>Piso desgastado na entrada do banheiro feminino do TIP em 20/03/2025;</t>
         </is>
       </c>
-      <c r="E36" t="inlineStr">
-        <is>
-          <t>foto01.jpg</t>
-        </is>
-      </c>
-      <c r="F36" t="inlineStr">
+      <c r="K36" t="inlineStr">
         <is>
           <t>Piso desgastado conforme evidência da foto 04.</t>
         </is>
@@ -2144,10 +2095,7 @@
       <c r="A37" t="n">
         <v>11</v>
       </c>
-      <c r="B37" t="n">
-        <v>1.8</v>
-      </c>
-      <c r="C37" t="inlineStr">
+      <c r="B37" t="inlineStr">
         <is>
           <t>Terminal de Caruaru (CAR)</t>
         </is>
@@ -2157,12 +2105,7 @@
           <t>Piso desgastado na entrada do banheiro feminino do TIP em 20/03/2025;</t>
         </is>
       </c>
-      <c r="E37" t="inlineStr">
-        <is>
-          <t>foto01.jpg</t>
-        </is>
-      </c>
-      <c r="F37" t="inlineStr">
+      <c r="K37" t="inlineStr">
         <is>
           <t>Piso desgastado conforme evidência da foto 04.</t>
         </is>
@@ -2172,10 +2115,7 @@
       <c r="A38" t="n">
         <v>11</v>
       </c>
-      <c r="B38" t="n">
-        <v>1.9</v>
-      </c>
-      <c r="C38" t="inlineStr">
+      <c r="B38" t="inlineStr">
         <is>
           <t>Terminal de Caruaru (CAR)</t>
         </is>
@@ -2185,12 +2125,7 @@
           <t>Piso desgastado na entrada do banheiro feminino do TIP em 20/03/2025;</t>
         </is>
       </c>
-      <c r="E38" t="inlineStr">
-        <is>
-          <t>foto01.jpg</t>
-        </is>
-      </c>
-      <c r="F38" t="inlineStr">
+      <c r="K38" t="inlineStr">
         <is>
           <t>Piso desgastado conforme evidência da foto 04.</t>
         </is>
@@ -2200,10 +2135,7 @@
       <c r="A39" t="n">
         <v>11</v>
       </c>
-      <c r="B39" t="n">
-        <v>1.1</v>
-      </c>
-      <c r="C39" t="inlineStr">
+      <c r="B39" t="inlineStr">
         <is>
           <t>Terminal de Caruaru (CAR)</t>
         </is>
@@ -2213,12 +2145,7 @@
           <t>Piso desgastado na entrada do banheiro feminino do TIP em 20/03/2025;</t>
         </is>
       </c>
-      <c r="E39" t="inlineStr">
-        <is>
-          <t>foto01.jpg</t>
-        </is>
-      </c>
-      <c r="F39" t="inlineStr">
+      <c r="K39" t="inlineStr">
         <is>
           <t>Piso desgastado conforme evidência da foto 04.</t>
         </is>
@@ -2228,10 +2155,7 @@
       <c r="A40" t="n">
         <v>11</v>
       </c>
-      <c r="B40" t="n">
-        <v>1.11</v>
-      </c>
-      <c r="C40" t="inlineStr">
+      <c r="B40" t="inlineStr">
         <is>
           <t>Terminal de Garanhuns (GAR)</t>
         </is>
@@ -2241,12 +2165,7 @@
           <t>Piso desgastado na entrada do banheiro feminino do TIP em 20/03/2025;</t>
         </is>
       </c>
-      <c r="E40" t="inlineStr">
-        <is>
-          <t>foto01.jpg</t>
-        </is>
-      </c>
-      <c r="F40" t="inlineStr">
+      <c r="K40" t="inlineStr">
         <is>
           <t>Piso desgastado conforme evidência da foto 04.</t>
         </is>
@@ -2256,10 +2175,7 @@
       <c r="A41" t="n">
         <v>11</v>
       </c>
-      <c r="B41" t="n">
-        <v>1.12</v>
-      </c>
-      <c r="C41" t="inlineStr">
+      <c r="B41" t="inlineStr">
         <is>
           <t>Terminal de Garanhuns (GAR)</t>
         </is>
@@ -2269,12 +2185,7 @@
           <t>Piso desgastado na entrada do banheiro feminino do TIP em 20/03/2025;</t>
         </is>
       </c>
-      <c r="E41" t="inlineStr">
-        <is>
-          <t>foto01.jpg</t>
-        </is>
-      </c>
-      <c r="F41" t="inlineStr">
+      <c r="K41" t="inlineStr">
         <is>
           <t>Piso desgastado conforme evidência da foto 04.</t>
         </is>
@@ -2284,10 +2195,7 @@
       <c r="A42" t="n">
         <v>11</v>
       </c>
-      <c r="B42" t="n">
-        <v>1.13</v>
-      </c>
-      <c r="C42" t="inlineStr">
+      <c r="B42" t="inlineStr">
         <is>
           <t>Terminal de Garanhuns (GAR)</t>
         </is>
@@ -2297,12 +2205,7 @@
           <t>Piso desgastado na entrada do banheiro feminino do TIP em 20/03/2025;</t>
         </is>
       </c>
-      <c r="E42" t="inlineStr">
-        <is>
-          <t>foto01.jpg</t>
-        </is>
-      </c>
-      <c r="F42" t="inlineStr">
+      <c r="K42" t="inlineStr">
         <is>
           <t>Piso desgastado conforme evidência da foto 04.</t>
         </is>
@@ -2312,10 +2215,7 @@
       <c r="A43" t="n">
         <v>11</v>
       </c>
-      <c r="B43" t="n">
-        <v>1.14</v>
-      </c>
-      <c r="C43" t="inlineStr">
+      <c r="B43" t="inlineStr">
         <is>
           <t>Terminal de Arcoverde (ARC)</t>
         </is>
@@ -2325,12 +2225,7 @@
           <t>Piso desgastado na entrada do banheiro feminino do TIP em 20/03/2025;</t>
         </is>
       </c>
-      <c r="E43" t="inlineStr">
-        <is>
-          <t>foto01.jpg</t>
-        </is>
-      </c>
-      <c r="F43" t="inlineStr">
+      <c r="K43" t="inlineStr">
         <is>
           <t>Piso desgastado conforme evidência da foto 04.</t>
         </is>
@@ -2340,10 +2235,7 @@
       <c r="A44" t="n">
         <v>11</v>
       </c>
-      <c r="B44" t="n">
-        <v>1.15</v>
-      </c>
-      <c r="C44" t="inlineStr">
+      <c r="B44" t="inlineStr">
         <is>
           <t>Terminal de Arcoverde (ARC)</t>
         </is>
@@ -2353,12 +2245,7 @@
           <t>Piso desgastado na entrada do banheiro feminino do TIP em 20/03/2025;</t>
         </is>
       </c>
-      <c r="E44" t="inlineStr">
-        <is>
-          <t>foto01.jpg</t>
-        </is>
-      </c>
-      <c r="F44" t="inlineStr">
+      <c r="K44" t="inlineStr">
         <is>
           <t>Piso desgastado conforme evidência da foto 04.</t>
         </is>
@@ -2368,10 +2255,7 @@
       <c r="A45" t="n">
         <v>11</v>
       </c>
-      <c r="B45" t="n">
-        <v>1.16</v>
-      </c>
-      <c r="C45" t="inlineStr">
+      <c r="B45" t="inlineStr">
         <is>
           <t>Terminal de Arcoverde (ARC)</t>
         </is>
@@ -2381,12 +2265,7 @@
           <t>Piso desgastado na entrada do banheiro feminino do TIP em 20/03/2025;</t>
         </is>
       </c>
-      <c r="E45" t="inlineStr">
-        <is>
-          <t>foto01.jpg</t>
-        </is>
-      </c>
-      <c r="F45" t="inlineStr">
+      <c r="K45" t="inlineStr">
         <is>
           <t>Piso desgastado conforme evidência da foto 04.</t>
         </is>
@@ -2396,10 +2275,7 @@
       <c r="A46" t="n">
         <v>11</v>
       </c>
-      <c r="B46" t="n">
-        <v>1.17</v>
-      </c>
-      <c r="C46" t="inlineStr">
+      <c r="B46" t="inlineStr">
         <is>
           <t>Terminal de Serra Talhada (SER)</t>
         </is>
@@ -2409,12 +2285,7 @@
           <t>Piso desgastado na entrada do banheiro feminino do TIP em 20/03/2025;</t>
         </is>
       </c>
-      <c r="E46" t="inlineStr">
-        <is>
-          <t>foto01.jpg</t>
-        </is>
-      </c>
-      <c r="F46" t="inlineStr">
+      <c r="K46" t="inlineStr">
         <is>
           <t>Piso desgastado conforme evidência da foto 04.</t>
         </is>
@@ -2424,10 +2295,7 @@
       <c r="A47" t="n">
         <v>11</v>
       </c>
-      <c r="B47" t="n">
-        <v>1.18</v>
-      </c>
-      <c r="C47" t="inlineStr">
+      <c r="B47" t="inlineStr">
         <is>
           <t>Terminal de Serra Talhada (SER)</t>
         </is>
@@ -2437,12 +2305,7 @@
           <t>Piso desgastado na entrada do banheiro feminino do TIP em 20/03/2025;</t>
         </is>
       </c>
-      <c r="E47" t="inlineStr">
-        <is>
-          <t>foto01.jpg</t>
-        </is>
-      </c>
-      <c r="F47" t="inlineStr">
+      <c r="K47" t="inlineStr">
         <is>
           <t>Piso desgastado conforme evidência da foto 04.</t>
         </is>
@@ -2452,10 +2315,7 @@
       <c r="A48" t="n">
         <v>11</v>
       </c>
-      <c r="B48" t="n">
-        <v>1.19</v>
-      </c>
-      <c r="C48" t="inlineStr">
+      <c r="B48" t="inlineStr">
         <is>
           <t>Terminal de Serra Talhada (SER)</t>
         </is>
@@ -2465,12 +2325,7 @@
           <t>Piso desgastado na entrada do banheiro feminino do TIP em 20/03/2025;</t>
         </is>
       </c>
-      <c r="E48" t="inlineStr">
-        <is>
-          <t>foto01.jpg</t>
-        </is>
-      </c>
-      <c r="F48" t="inlineStr">
+      <c r="K48" t="inlineStr">
         <is>
           <t>Piso desgastado conforme evidência da foto 04.</t>
         </is>
@@ -2480,10 +2335,7 @@
       <c r="A49" t="n">
         <v>11</v>
       </c>
-      <c r="B49" t="n">
-        <v>1.2</v>
-      </c>
-      <c r="C49" t="inlineStr">
+      <c r="B49" t="inlineStr">
         <is>
           <t>Terminal de Serra Talhada (SER)</t>
         </is>
@@ -2493,12 +2345,7 @@
           <t>Piso desgastado na entrada do banheiro feminino do TIP em 20/03/2025;</t>
         </is>
       </c>
-      <c r="E49" t="inlineStr">
-        <is>
-          <t>foto01.jpg</t>
-        </is>
-      </c>
-      <c r="F49" t="inlineStr">
+      <c r="K49" t="inlineStr">
         <is>
           <t>Piso desgastado conforme evidência da foto 04.</t>
         </is>
@@ -2508,10 +2355,7 @@
       <c r="A50" t="n">
         <v>11</v>
       </c>
-      <c r="B50" t="n">
-        <v>1.21</v>
-      </c>
-      <c r="C50" t="inlineStr">
+      <c r="B50" t="inlineStr">
         <is>
           <t>Terminal de Serra Talhada (SER)</t>
         </is>
@@ -2521,12 +2365,7 @@
           <t>Piso desgastado na entrada do banheiro feminino do TIP em 20/03/2025;</t>
         </is>
       </c>
-      <c r="E50" t="inlineStr">
-        <is>
-          <t>foto01.jpg</t>
-        </is>
-      </c>
-      <c r="F50" t="inlineStr">
+      <c r="K50" t="inlineStr">
         <is>
           <t>Piso desgastado conforme evidência da foto 04.</t>
         </is>
@@ -2536,10 +2375,7 @@
       <c r="A51" t="n">
         <v>11</v>
       </c>
-      <c r="B51" t="n">
-        <v>1.22</v>
-      </c>
-      <c r="C51" t="inlineStr">
+      <c r="B51" t="inlineStr">
         <is>
           <t>Terminal de Serra Talhada (SER)</t>
         </is>
@@ -2549,12 +2385,7 @@
           <t>Piso desgastado na entrada do banheiro feminino do TIP em 20/03/2025;</t>
         </is>
       </c>
-      <c r="E51" t="inlineStr">
-        <is>
-          <t>foto01.jpg</t>
-        </is>
-      </c>
-      <c r="F51" t="inlineStr">
+      <c r="K51" t="inlineStr">
         <is>
           <t>Piso desgastado conforme evidência da foto 04.</t>
         </is>
@@ -2564,10 +2395,7 @@
       <c r="A52" t="n">
         <v>11</v>
       </c>
-      <c r="B52" t="n">
-        <v>1.23</v>
-      </c>
-      <c r="C52" t="inlineStr">
+      <c r="B52" t="inlineStr">
         <is>
           <t>Terminal de Serra Talhada (SER)</t>
         </is>
@@ -2577,12 +2405,7 @@
           <t>Piso desgastado na entrada do banheiro feminino do TIP em 20/03/2025;</t>
         </is>
       </c>
-      <c r="E52" t="inlineStr">
-        <is>
-          <t>foto01.jpg</t>
-        </is>
-      </c>
-      <c r="F52" t="inlineStr">
+      <c r="K52" t="inlineStr">
         <is>
           <t>Piso desgastado conforme evidência da foto 04.</t>
         </is>
@@ -2592,10 +2415,7 @@
       <c r="A53" t="n">
         <v>11</v>
       </c>
-      <c r="B53" t="n">
-        <v>1.24</v>
-      </c>
-      <c r="C53" t="inlineStr">
+      <c r="B53" t="inlineStr">
         <is>
           <t>Terminal de Serra Talhada (SER)</t>
         </is>
@@ -2605,12 +2425,7 @@
           <t>Piso desgastado na entrada do banheiro feminino do TIP em 20/03/2025;</t>
         </is>
       </c>
-      <c r="E53" t="inlineStr">
-        <is>
-          <t>foto01.jpg</t>
-        </is>
-      </c>
-      <c r="F53" t="inlineStr">
+      <c r="K53" t="inlineStr">
         <is>
           <t>Piso desgastado conforme evidência da foto 04.</t>
         </is>
@@ -2620,10 +2435,7 @@
       <c r="A54" t="n">
         <v>12</v>
       </c>
-      <c r="B54" t="n">
-        <v>1</v>
-      </c>
-      <c r="C54" t="inlineStr">
+      <c r="B54" t="inlineStr">
         <is>
           <t>Terminal do Recife (TIP)</t>
         </is>
@@ -2633,12 +2445,7 @@
           <t>Piso desgastado na entrada do banheiro feminino do TIP em 20/03/2025;</t>
         </is>
       </c>
-      <c r="E54" t="inlineStr">
-        <is>
-          <t>foto01.jpg;foto02.jpg</t>
-        </is>
-      </c>
-      <c r="F54" t="inlineStr">
+      <c r="K54" t="inlineStr">
         <is>
           <t xml:space="preserve">Piso desgastado conforme evidência da foto 04.;Segunda legenda qualquer coisa. </t>
         </is>
@@ -2648,10 +2455,7 @@
       <c r="A55" t="n">
         <v>12</v>
       </c>
-      <c r="B55" t="n">
-        <v>1.1</v>
-      </c>
-      <c r="C55" t="inlineStr">
+      <c r="B55" t="inlineStr">
         <is>
           <t>Terminal do Recife (TIP)</t>
         </is>
@@ -2661,12 +2465,7 @@
           <t>Piso desgastado na entrada do banheiro feminino do TIP em 20/03/2025;</t>
         </is>
       </c>
-      <c r="E55" t="inlineStr">
-        <is>
-          <t>foto01.jpg</t>
-        </is>
-      </c>
-      <c r="F55" t="inlineStr">
+      <c r="K55" t="inlineStr">
         <is>
           <t xml:space="preserve">Piso desgastado conforme evidência da foto 04.;Segunda legenda qualquer coisa. </t>
         </is>
@@ -2676,10 +2475,7 @@
       <c r="A56" t="n">
         <v>12</v>
       </c>
-      <c r="B56" t="n">
-        <v>1.2</v>
-      </c>
-      <c r="C56" t="inlineStr">
+      <c r="B56" t="inlineStr">
         <is>
           <t>Terminal do Recife (TIP)</t>
         </is>
@@ -2689,7 +2485,7 @@
           <t>Piso desgastado na entrada do banheiro feminino do TIP em 20/03/2025;</t>
         </is>
       </c>
-      <c r="F56" t="inlineStr">
+      <c r="K56" t="inlineStr">
         <is>
           <t xml:space="preserve">Piso desgastado conforme evidência da foto 04.;Segunda legenda qualquer coisa. </t>
         </is>
@@ -2699,10 +2495,7 @@
       <c r="A57" t="n">
         <v>12</v>
       </c>
-      <c r="B57" t="n">
-        <v>1.3</v>
-      </c>
-      <c r="C57" t="inlineStr">
+      <c r="B57" t="inlineStr">
         <is>
           <t>Terminal do Recife (TIP)</t>
         </is>
@@ -2712,12 +2505,7 @@
           <t>Piso desgastado na entrada do banheiro feminino do TIP em 20/03/2025;</t>
         </is>
       </c>
-      <c r="E57" t="inlineStr">
-        <is>
-          <t>foto01.jpg;foto02.jpg;foto01.jpg;foto02.jpg;foto01.jpg;foto02.jpg</t>
-        </is>
-      </c>
-      <c r="F57" t="inlineStr">
+      <c r="K57" t="inlineStr">
         <is>
           <t xml:space="preserve">Piso desgastado conforme evidência da foto 04.;Segunda legenda qualquer coisa. ;Piso desgastado conforme evidência da foto 04.;Segunda legenda qualquer coisa. ;Piso desgastado conforme evidência da foto 04.;Segunda legenda qualquer coisa. </t>
         </is>
@@ -2727,10 +2515,7 @@
       <c r="A58" t="n">
         <v>12</v>
       </c>
-      <c r="B58" t="n">
-        <v>1.4</v>
-      </c>
-      <c r="C58" t="inlineStr">
+      <c r="B58" t="inlineStr">
         <is>
           <t>Terminal do Recife (TIP)</t>
         </is>
@@ -2740,12 +2525,7 @@
           <t>Piso desgastado na entrada do banheiro feminino do TIP em 20/03/2025;</t>
         </is>
       </c>
-      <c r="E58" t="inlineStr">
-        <is>
-          <t>foto01.jpg;foto02.jpg</t>
-        </is>
-      </c>
-      <c r="F58" t="inlineStr">
+      <c r="K58" t="inlineStr">
         <is>
           <t xml:space="preserve">Piso desgastado conforme evidência da foto 04.;Segunda legenda qualquer coisa. </t>
         </is>
@@ -2755,10 +2535,7 @@
       <c r="A59" t="n">
         <v>12</v>
       </c>
-      <c r="B59" t="n">
-        <v>1.5</v>
-      </c>
-      <c r="C59" t="inlineStr">
+      <c r="B59" t="inlineStr">
         <is>
           <t>Terminal de Serra Talhada (SER)</t>
         </is>
@@ -2768,12 +2545,7 @@
           <t>Piso desgastado na entrada do banheiro feminino do TIP em 20/03/2025;</t>
         </is>
       </c>
-      <c r="E59" t="inlineStr">
-        <is>
-          <t>foto01.jpg;foto02.jpg</t>
-        </is>
-      </c>
-      <c r="F59" t="inlineStr">
+      <c r="K59" t="inlineStr">
         <is>
           <t xml:space="preserve">Piso desgastado conforme evidência da foto 04.;Segunda legenda qualquer coisa. </t>
         </is>
@@ -2783,10 +2555,7 @@
       <c r="A60" t="n">
         <v>12</v>
       </c>
-      <c r="B60" t="n">
-        <v>1.6</v>
-      </c>
-      <c r="C60" t="inlineStr">
+      <c r="B60" t="inlineStr">
         <is>
           <t>Terminal de Serra Talhada (SER)</t>
         </is>
@@ -2801,10 +2570,7 @@
       <c r="A61" t="n">
         <v>12</v>
       </c>
-      <c r="B61" t="n">
-        <v>1.7</v>
-      </c>
-      <c r="C61" t="inlineStr">
+      <c r="B61" t="inlineStr">
         <is>
           <t>Terminal de Serra Talhada (SER)</t>
         </is>
@@ -2814,12 +2580,7 @@
           <t>Piso desgastado na entrada do banheiro feminino do TIP em 20/03/2025;</t>
         </is>
       </c>
-      <c r="E61" t="inlineStr">
-        <is>
-          <t>foto01.jpg</t>
-        </is>
-      </c>
-      <c r="F61" t="inlineStr">
+      <c r="K61" t="inlineStr">
         <is>
           <t>Piso desgastado conforme evidência da foto 04.</t>
         </is>
@@ -2829,10 +2590,7 @@
       <c r="A62" t="n">
         <v>12</v>
       </c>
-      <c r="B62" t="n">
-        <v>1.8</v>
-      </c>
-      <c r="C62" t="inlineStr">
+      <c r="B62" t="inlineStr">
         <is>
           <t>Terminal de Serra Talhada (SER)</t>
         </is>
@@ -2847,10 +2605,7 @@
       <c r="A63" t="n">
         <v>12</v>
       </c>
-      <c r="B63" t="n">
-        <v>1.9</v>
-      </c>
-      <c r="C63" t="inlineStr">
+      <c r="B63" t="inlineStr">
         <is>
           <t>Terminal de Arcoverde (ARC)</t>
         </is>
@@ -2860,12 +2615,7 @@
           <t>Piso desgastado na entrada do banheiro feminino do TIP em 20/03/2025;</t>
         </is>
       </c>
-      <c r="E63" t="inlineStr">
-        <is>
-          <t>foto01.jpg;foto02.jpg</t>
-        </is>
-      </c>
-      <c r="F63" t="inlineStr">
+      <c r="K63" t="inlineStr">
         <is>
           <t xml:space="preserve">Piso desgastado conforme evidência da foto 04.;Segunda legenda qualquer coisa. </t>
         </is>
@@ -2875,10 +2625,7 @@
       <c r="A64" t="n">
         <v>12</v>
       </c>
-      <c r="B64" t="n">
-        <v>1.1</v>
-      </c>
-      <c r="C64" t="inlineStr">
+      <c r="B64" t="inlineStr">
         <is>
           <t>Terminal de Arcoverde (ARC)</t>
         </is>
@@ -2888,12 +2635,7 @@
           <t>Piso desgastado na entrada do banheiro feminino do TIP em 20/03/2025;</t>
         </is>
       </c>
-      <c r="E64" t="inlineStr">
-        <is>
-          <t>foto01.jpg;foto02.jpg</t>
-        </is>
-      </c>
-      <c r="F64" t="inlineStr">
+      <c r="K64" t="inlineStr">
         <is>
           <t xml:space="preserve">Piso desgastado conforme evidência da foto 04.;Segunda legenda qualquer coisa. </t>
         </is>
@@ -2903,10 +2645,7 @@
       <c r="A65" t="n">
         <v>12</v>
       </c>
-      <c r="B65" t="n">
-        <v>1.11</v>
-      </c>
-      <c r="C65" t="inlineStr">
+      <c r="B65" t="inlineStr">
         <is>
           <t>Terminal de Arcoverde (ARC)</t>
         </is>
@@ -2916,12 +2655,7 @@
           <t>Piso desgastado na entrada do banheiro feminino do TIP em 20/03/2025;</t>
         </is>
       </c>
-      <c r="E65" t="inlineStr">
-        <is>
-          <t>foto01.jpg;foto02.jpg</t>
-        </is>
-      </c>
-      <c r="F65" t="inlineStr">
+      <c r="K65" t="inlineStr">
         <is>
           <t xml:space="preserve">Piso desgastado conforme evidência da foto 04.;Segunda legenda qualquer coisa. </t>
         </is>
@@ -2931,10 +2665,7 @@
       <c r="A66" t="n">
         <v>12</v>
       </c>
-      <c r="B66" t="n">
-        <v>1.12</v>
-      </c>
-      <c r="C66" t="inlineStr">
+      <c r="B66" t="inlineStr">
         <is>
           <t>Terminal de Arcoverde (ARC)</t>
         </is>
@@ -2944,12 +2675,7 @@
           <t>Piso desgastado na entrada do banheiro feminino do TIP em 20/03/2025;</t>
         </is>
       </c>
-      <c r="E66" t="inlineStr">
-        <is>
-          <t>foto01.jpg;foto02.jpg</t>
-        </is>
-      </c>
-      <c r="F66" t="inlineStr">
+      <c r="K66" t="inlineStr">
         <is>
           <t xml:space="preserve">Piso desgastado conforme evidência da foto 04.;Segunda legenda qualquer coisa. </t>
         </is>
@@ -2959,10 +2685,7 @@
       <c r="A67" t="n">
         <v>12</v>
       </c>
-      <c r="B67" t="n">
-        <v>1.13</v>
-      </c>
-      <c r="C67" t="inlineStr">
+      <c r="B67" t="inlineStr">
         <is>
           <t>Terminal de Caruaru (CAR)</t>
         </is>
@@ -2972,12 +2695,7 @@
           <t>Piso desgastado na entrada do banheiro feminino do TIP em 20/03/2025;</t>
         </is>
       </c>
-      <c r="E67" t="inlineStr">
-        <is>
-          <t>foto01.jpg;foto02.jpg</t>
-        </is>
-      </c>
-      <c r="F67" t="inlineStr">
+      <c r="K67" t="inlineStr">
         <is>
           <t xml:space="preserve">Piso desgastado conforme evidência da foto 04.;Segunda legenda qualquer coisa. </t>
         </is>
@@ -2987,10 +2705,7 @@
       <c r="A68" t="n">
         <v>12</v>
       </c>
-      <c r="B68" t="n">
-        <v>1.14</v>
-      </c>
-      <c r="C68" t="inlineStr">
+      <c r="B68" t="inlineStr">
         <is>
           <t>Terminal de Caruaru (CAR)</t>
         </is>
@@ -3000,12 +2715,7 @@
           <t>Piso desgastado na entrada do banheiro feminino do TIP em 20/03/2025;</t>
         </is>
       </c>
-      <c r="E68" t="inlineStr">
-        <is>
-          <t>foto01.jpg;foto02.jpg</t>
-        </is>
-      </c>
-      <c r="F68" t="inlineStr">
+      <c r="K68" t="inlineStr">
         <is>
           <t xml:space="preserve">Piso desgastado conforme evidência da foto 04.;Segunda legenda qualquer coisa. </t>
         </is>
@@ -3015,10 +2725,7 @@
       <c r="A69" t="n">
         <v>12</v>
       </c>
-      <c r="B69" t="n">
-        <v>1.15</v>
-      </c>
-      <c r="C69" t="inlineStr">
+      <c r="B69" t="inlineStr">
         <is>
           <t>Terminal de Caruaru (CAR)</t>
         </is>
@@ -3028,12 +2735,7 @@
           <t>Piso desgastado na entrada do banheiro feminino do TIP em 20/03/2025;</t>
         </is>
       </c>
-      <c r="E69" t="inlineStr">
-        <is>
-          <t>foto01.jpg;foto02.jpg</t>
-        </is>
-      </c>
-      <c r="F69" t="inlineStr">
+      <c r="K69" t="inlineStr">
         <is>
           <t xml:space="preserve">Piso desgastado conforme evidência da foto 04.;Segunda legenda qualquer coisa. </t>
         </is>
@@ -3043,10 +2745,7 @@
       <c r="A70" t="n">
         <v>12</v>
       </c>
-      <c r="B70" t="n">
-        <v>1.16</v>
-      </c>
-      <c r="C70" t="inlineStr">
+      <c r="B70" t="inlineStr">
         <is>
           <t>Terminal de Caruaru (CAR)</t>
         </is>
@@ -3056,12 +2755,7 @@
           <t>Piso desgastado na entrada do banheiro feminino do TIP em 20/03/2025;</t>
         </is>
       </c>
-      <c r="E70" t="inlineStr">
-        <is>
-          <t>foto01.jpg;foto02.jpg</t>
-        </is>
-      </c>
-      <c r="F70" t="inlineStr">
+      <c r="K70" t="inlineStr">
         <is>
           <t xml:space="preserve">Piso desgastado conforme evidência da foto 04.;Segunda legenda qualquer coisa. </t>
         </is>
@@ -3071,10 +2765,7 @@
       <c r="A71" t="n">
         <v>12</v>
       </c>
-      <c r="B71" t="n">
-        <v>1.17</v>
-      </c>
-      <c r="C71" t="inlineStr">
+      <c r="B71" t="inlineStr">
         <is>
           <t>Terminal de Caruaru (CAR)</t>
         </is>
@@ -3084,401 +2775,569 @@
           <t>Piso desgastado na entrada do banheiro feminino do TIP em 20/03/2025;</t>
         </is>
       </c>
-      <c r="E71" t="inlineStr">
-        <is>
-          <t>foto01.jpg;foto02.jpg</t>
-        </is>
-      </c>
-      <c r="F71" t="inlineStr">
+      <c r="K71" t="inlineStr">
         <is>
           <t xml:space="preserve">Piso desgastado conforme evidência da foto 04.;Segunda legenda qualquer coisa. </t>
         </is>
       </c>
     </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:E13"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="2" t="inlineStr">
-        <is>
-          <t>ID da Fiscalização</t>
-        </is>
-      </c>
-      <c r="B1" s="2" t="inlineStr">
-        <is>
-          <t>Terminal</t>
-        </is>
-      </c>
-      <c r="C1" s="2" t="inlineStr">
-        <is>
-          <t>Observações</t>
-        </is>
-      </c>
-      <c r="D1" s="2" t="inlineStr">
-        <is>
-          <t>Foto</t>
-        </is>
-      </c>
-      <c r="E1" s="2" t="inlineStr">
-        <is>
-          <t>Legenda da Foto</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="n">
-        <v>1</v>
-      </c>
-      <c r="B2" t="inlineStr">
+    <row r="72">
+      <c r="A72" t="n">
+        <v>13</v>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>Terminal de Caruaru (CAR)</t>
+        </is>
+      </c>
+      <c r="D72" t="inlineStr">
+        <is>
+          <t>Piso desgastado na entrada do banheiro feminino do TIP em 20/03/2025;</t>
+        </is>
+      </c>
+      <c r="K72" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Piso desgastado conforme evidência da foto 04.;Segunda legenda qualquer coisa. </t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="n">
+        <v>13</v>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>Terminal de Arcoverde (ARC)</t>
+        </is>
+      </c>
+      <c r="D73" t="inlineStr">
+        <is>
+          <t>Piso desgastado na entrada do banheiro feminino do TIP em 20/03/2025;</t>
+        </is>
+      </c>
+      <c r="K73" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Piso desgastado conforme evidência da foto 04.;Segunda legenda qualquer coisa. </t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="n">
+        <v>13</v>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>Terminal de Serra Talhada (SER)</t>
+        </is>
+      </c>
+      <c r="D74" t="inlineStr">
+        <is>
+          <t>Piso desgastado na entrada do banheiro feminino do TIP em 20/03/2025;</t>
+        </is>
+      </c>
+      <c r="K74" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Piso desgastado conforme evidência da foto 04.;Segunda legenda qualquer coisa. </t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="n">
+        <v>13</v>
+      </c>
+      <c r="B75" t="inlineStr">
         <is>
           <t>Terminal do Recife (TIP)</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>Lorem ipsum lorem pisum ipsum lorem pisum ipsum lorem pisum ipsum lorem pisum ipsum lorem pisum ipsum lorem pisum ipsum lorem pisum ipsum lorem pisum ipsum lorem pisum ipsum lorem pisum.</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>foto01.jpg</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>Viga do terminal não posicionada corretamente.</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="n">
-        <v>1</v>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>Terminal de Caruaru</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>Lorem ipsum lorem pisum ipsum lorem pisum ipsum lorem pisum ipsum lorem pisum ipsum lorem pisum ipsum lorem pisum ipsum lorem pisum ipsum lorem pisum ipsum lorem pisum ipsum lorem pisum.</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="n">
-        <v>11</v>
-      </c>
-      <c r="B4" t="inlineStr">
+      <c r="D75" t="inlineStr">
+        <is>
+          <t>Piso desgastado na entrada do banheiro feminino do TIP em 20/03/2025;</t>
+        </is>
+      </c>
+      <c r="K75" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Piso desgastado conforme evidência da foto 04.;Segunda legenda qualquer coisa. </t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="n">
+        <v>13</v>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>Terminal de Garanhuns (GAR)</t>
+        </is>
+      </c>
+      <c r="D76" t="inlineStr">
+        <is>
+          <t>Piso desgastado na entrada do banheiro feminino do TIP em 20/03/2025;</t>
+        </is>
+      </c>
+      <c r="K76" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Piso desgastado conforme evidência da foto 04.;Segunda legenda qualquer coisa. </t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="n">
+        <v>13</v>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>Terminal de Caruaru (CAR)</t>
+        </is>
+      </c>
+      <c r="D77" t="inlineStr">
+        <is>
+          <t>Piso desgastado na entrada do banheiro feminino do TIP em 20/03/2025;</t>
+        </is>
+      </c>
+      <c r="K77" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Piso desgastado conforme evidência da foto 04.;Segunda legenda qualquer coisa. </t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="n">
+        <v>13</v>
+      </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>Terminal de Caruaru (CAR)</t>
+        </is>
+      </c>
+      <c r="D78" t="inlineStr">
+        <is>
+          <t>Piso desgastado na entrada do banheiro feminino do TIP em 20/03/2025;</t>
+        </is>
+      </c>
+      <c r="K78" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Piso desgastado conforme evidência da foto 04.;Segunda legenda qualquer coisa. </t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="n">
+        <v>14</v>
+      </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>Terminal de Caruaru (CAR)</t>
+        </is>
+      </c>
+      <c r="D79" t="inlineStr">
+        <is>
+          <t>Piso desgastado na entrada do banheiro feminino do TIP em 20/03/2025;</t>
+        </is>
+      </c>
+      <c r="K79" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Piso desgastado conforme evidência da foto 04.;Segunda legenda qualquer coisa. </t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="n">
+        <v>14</v>
+      </c>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>Terminal de Garanhuns (GAR)</t>
+        </is>
+      </c>
+      <c r="D80" t="inlineStr">
+        <is>
+          <t>Piso desgastado na entrada do banheiro feminino do TIP em 20/03/2025;</t>
+        </is>
+      </c>
+      <c r="K80" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Piso desgastado conforme evidência da foto 04.;Segunda legenda qualquer coisa. </t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="n">
+        <v>14</v>
+      </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>Terminal de Serra Talhada (SER)</t>
+        </is>
+      </c>
+      <c r="D81" t="inlineStr">
+        <is>
+          <t>Piso desgastado na entrada do banheiro feminino do TIP em 20/03/2025;</t>
+        </is>
+      </c>
+      <c r="K81" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Piso desgastado conforme evidência da foto 04.;Segunda legenda qualquer coisa. </t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="n">
+        <v>14</v>
+      </c>
+      <c r="B82" t="inlineStr">
+        <is>
+          <t>Terminal de Arcoverde (ARC)</t>
+        </is>
+      </c>
+      <c r="D82" t="inlineStr">
+        <is>
+          <t>Piso desgastado na entrada do banheiro feminino do TIP em 20/03/2025;</t>
+        </is>
+      </c>
+      <c r="K82" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Piso desgastado conforme evidência da foto 04.;Segunda legenda qualquer coisa. </t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="n">
+        <v>14</v>
+      </c>
+      <c r="B83" t="inlineStr">
+        <is>
+          <t>Terminal de Arcoverde (ARC)</t>
+        </is>
+      </c>
+      <c r="D83" t="inlineStr">
+        <is>
+          <t>Piso desgastado na entrada do banheiro feminino do TIP em 20/03/2025;</t>
+        </is>
+      </c>
+      <c r="K83" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Piso desgastado conforme evidência da foto 04.;Segunda legenda qualquer coisa. </t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="n">
+        <v>14</v>
+      </c>
+      <c r="B84" t="inlineStr">
         <is>
           <t>Terminal do Recife (TIP)</t>
         </is>
       </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>Durante a fiscalização, foi observada a presença de cidadãos que ficaram fiscalizando o serviço conforme o andamento do mesmo. Precisamos mobilizar uma equipe que fiscalize os agentes e os cidadãos em campo.</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>foto01.jpg</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>Viga do terminal não posicionada corretamente.</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="n">
-        <v>11</v>
-      </c>
-      <c r="B5" t="inlineStr">
+      <c r="D84" t="inlineStr">
+        <is>
+          <t>Piso desgastado na entrada do banheiro feminino do TIP em 20/03/2025;</t>
+        </is>
+      </c>
+      <c r="K84" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Piso desgastado conforme evidência da foto 04.;Segunda legenda qualquer coisa. </t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="n">
+        <v>14</v>
+      </c>
+      <c r="B85" t="inlineStr">
         <is>
           <t>Terminal de Caruaru (CAR)</t>
         </is>
       </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>Durante a fiscalização, foi observada a presença de cidadãos que ficaram fiscalizando o serviço conforme o andamento do mesmo. Precisamos mobilizar uma equipe que fiscalize os agentes e os cidadãos em campo.</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="n">
-        <v>11</v>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>Terminal de Arcoverde (ARC)</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>Durante a fiscalização, foi observada a presença de cidadãos que ficaram fiscalizando o serviço conforme o andamento do mesmo. Precisamos mobilizar uma equipe que fiscalize os agentes e os cidadãos em campo.</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="n">
-        <v>11</v>
-      </c>
-      <c r="B7" t="inlineStr">
+      <c r="D85" t="inlineStr">
+        <is>
+          <t>Piso desgastado na entrada do banheiro feminino do TIP em 20/03/2025;</t>
+        </is>
+      </c>
+      <c r="K85" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Piso desgastado conforme evidência da foto 04.;Segunda legenda qualquer coisa. </t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="n">
+        <v>14</v>
+      </c>
+      <c r="B86" t="inlineStr">
+        <is>
+          <t>Terminal de Caruaru (CAR)</t>
+        </is>
+      </c>
+      <c r="D86" t="inlineStr">
+        <is>
+          <t>Piso desgastado na entrada do banheiro feminino do TIP em 20/03/2025;</t>
+        </is>
+      </c>
+      <c r="K86" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Piso desgastado conforme evidência da foto 04.;Segunda legenda qualquer coisa. </t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="n">
+        <v>14</v>
+      </c>
+      <c r="B87" t="inlineStr">
+        <is>
+          <t>Terminal de Caruaru (CAR)</t>
+        </is>
+      </c>
+      <c r="D87" t="inlineStr">
+        <is>
+          <t>Piso desgastado na entrada do banheiro feminino do TIP em 20/03/2025;</t>
+        </is>
+      </c>
+      <c r="K87" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Piso desgastado conforme evidência da foto 04.;Segunda legenda qualquer coisa. </t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="n">
+        <v>14</v>
+      </c>
+      <c r="B88" t="inlineStr">
+        <is>
+          <t>Terminal de Caruaru (CAR)</t>
+        </is>
+      </c>
+      <c r="D88" t="inlineStr">
+        <is>
+          <t>Piso desgastado na entrada do banheiro feminino do TIP em 20/03/2025;</t>
+        </is>
+      </c>
+      <c r="K88" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Piso desgastado conforme evidência da foto 04.;Segunda legenda qualquer coisa. </t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="n">
+        <v>15</v>
+      </c>
+      <c r="B89" t="inlineStr">
+        <is>
+          <t>Terminal de Caruaru (CAR)</t>
+        </is>
+      </c>
+      <c r="D89" t="inlineStr">
+        <is>
+          <t>Piso desgastado na entrada do banheiro feminino do TIP em 20/03/2025;</t>
+        </is>
+      </c>
+      <c r="K89" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Piso desgastado conforme evidência da foto 04.;Segunda legenda qualquer coisa. </t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="n">
+        <v>15</v>
+      </c>
+      <c r="B90" t="inlineStr">
+        <is>
+          <t>Terminal de Caruaru (CAR)</t>
+        </is>
+      </c>
+      <c r="D90" t="inlineStr">
+        <is>
+          <t>Piso desgastado na entrada do banheiro feminino do TIP em 20/03/2025;</t>
+        </is>
+      </c>
+      <c r="K90" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Piso desgastado conforme evidência da foto 04.;Segunda legenda qualquer coisa. </t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="n">
+        <v>15</v>
+      </c>
+      <c r="B91" t="inlineStr">
         <is>
           <t>Terminal de Serra Talhada (SER)</t>
         </is>
       </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>Durante a fiscalização, foi observada a presença de cidadãos que ficaram fiscalizando o serviço conforme o andamento do mesmo. Precisamos mobilizar uma equipe que fiscalize os agentes e os cidadãos em campo.</t>
-        </is>
-      </c>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t>foto01.jpg;foto02.jpg</t>
-        </is>
-      </c>
-      <c r="E7" t="inlineStr">
-        <is>
-          <t>Viga do terminal não posicionada corretamente.;Piso desgastado na entrada do banheiro feminino do TIP em 20/03/2025.;</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="n">
-        <v>11</v>
-      </c>
-      <c r="B8" t="inlineStr">
+      <c r="D91" t="inlineStr">
+        <is>
+          <t>Piso desgastado na entrada do banheiro feminino do TIP em 20/03/2025;</t>
+        </is>
+      </c>
+      <c r="K91" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Piso desgastado conforme evidência da foto 04.;Segunda legenda qualquer coisa. </t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="n">
+        <v>17</v>
+      </c>
+      <c r="B92" t="inlineStr">
+        <is>
+          <t>Terminal de Recife (TIP)</t>
+        </is>
+      </c>
+      <c r="C92" t="inlineStr">
+        <is>
+          <t>TIP_2025_01;TIP_2025_02;TIP_2025_03;TIP_2025_04;TIP_2025_05</t>
+        </is>
+      </c>
+      <c r="D92" t="inlineStr">
+        <is>
+          <t>Base do suporte da sinalização em braile enferrujada e desatualizada na área de embarque e desembarque do Terminal de Recife (TIP), conforme evidenciado nas Fotos 01 e 02, a seguir.; Falta de manutenção adequada no banheiro masculino para PCD localizado no térreo do Terminal de Recife (TIP), conforme detalhado.;Saboneteira ausente, a seguir na Fotos 03 e 04.; Pia com vazamento, conforme a Fotos 03 e 04.;Fachada interna necessitando de pintura do Terminal de Recife (TIP), conforme evidenciado na Fotos 05 e 06, a seguir.</t>
+        </is>
+      </c>
+      <c r="H92" t="inlineStr">
+        <is>
+          <t>LOREM IPSUM;LOREM IPSUM; lalala;hahaha;pipipip</t>
+        </is>
+      </c>
+      <c r="I92" t="inlineStr">
+        <is>
+          <t>LOREM IPSUM</t>
+        </is>
+      </c>
+      <c r="J92" t="inlineStr">
+        <is>
+          <t>LOREM IPSUM;LOREM IPSUM</t>
+        </is>
+      </c>
+      <c r="K92" t="inlineStr">
+        <is>
+          <t>Suporte da sinalização em braile enferrujada do Terminal do Recife em 30/09/2025:sinalização em braile enferrujada do Terminal do Recife em 30/09/2025;Pia com vazamento e saboneteira quebrada no banheiro do térreo masculino para PCD do Terminal de Recife em 30/09/2025:vazamento e saboneteira quebrada no banheiro do térreo masculino para PCD do Terminal de Recife ;Pintura da fachada  do pátio interno desgastada no Terminal de Recife em 30/09/202510/11/2025:fachada do pátio interno desgastada no Terminal de Recife em 30/09/2025</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="n">
+        <v>17</v>
+      </c>
+      <c r="B93" t="inlineStr">
+        <is>
+          <t>Terminal de Caruaru (CAR)</t>
+        </is>
+      </c>
+      <c r="C93" t="inlineStr">
+        <is>
+          <t>CAR_2025_00;CAR_2025_08;CAR_2025_10</t>
+        </is>
+      </c>
+      <c r="D93" t="inlineStr">
+        <is>
+          <t>Placas do teto do terminal apresentando descolamentos no pátio de manobras do Terminal de Caruaru, conforme evidenciado na Foto 07 e foto 08, a seguir.; Viga apresentando rachaduras próximo a juntas da testeira necessitando de reparo estrutural no pátio de manobras do Terminal de Caruaru, conforme evidenciado na Fotos 09 e 10, a seguir.</t>
+        </is>
+      </c>
+      <c r="H93" t="inlineStr">
+        <is>
+          <t>LOREM IPSUM;LOREM IPSUM</t>
+        </is>
+      </c>
+      <c r="I93" t="inlineStr">
+        <is>
+          <t>LOREM IPSUM</t>
+        </is>
+      </c>
+      <c r="J93" t="inlineStr">
+        <is>
+          <t>LOREM IPSUM;LOREM IPSUM</t>
+        </is>
+      </c>
+      <c r="K93" t="inlineStr">
+        <is>
+          <t>Placas descoladas no Terminal de Caruaru em 25/09/2025.;Placas descoladas no Terminal de Caruaru em 25/09/2025.;Rachaduras próximas à junta de dilatação na testeira do pátio de manobras no Terminal de Caruaru em 25/09/2025.;Detalhe das rachaduras na testeira do pátio de manobras no Terminal de Caruaru em 25/09/2025.</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="n">
+        <v>17</v>
+      </c>
+      <c r="B94" t="inlineStr">
         <is>
           <t>Terminal de Garanhuns (GAR)</t>
         </is>
       </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>Durante a fiscalização, foi observada a presença de cidadãos que ficaram fiscalizando o serviço conforme o andamento do mesmo. Precisamos mobilizar uma equipe que fiscalize os agentes e os cidadãos em campo.</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="n">
-        <v>12</v>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>Terminal do Recife (TIP)</t>
-        </is>
-      </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>Durante a fiscalização, foi observada a presença de cidadãos que ficaram fiscalizando o serviço conforme o andamento do mesmo. Precisamos mobilizar uma equipe que fiscalize os agentes e os cidadãos em campo.</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="n">
-        <v>12</v>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>Terminal de Arcoverde (ARC)</t>
-        </is>
-      </c>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t>Durante a fiscalização, foi observada a presença de cidadãos que ficaram fiscalizando o serviço conforme o andamento do mesmo. Precisamos mobilizar uma equipe que fiscalize os agentes e os cidadãos em campo.</t>
-        </is>
-      </c>
-      <c r="D10" t="inlineStr">
-        <is>
-          <t>foto01.jpg;foto02.jpg</t>
-        </is>
-      </c>
-      <c r="E10" t="inlineStr">
-        <is>
-          <t>Viga do terminal não posicionada corretamente.;Piso desgastado na entrada do banheiro feminino do TIP em 20/03/2025.;</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="n">
-        <v>12</v>
-      </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>Terminal de Serra Talhada (SER)</t>
-        </is>
-      </c>
-      <c r="C11" t="inlineStr">
-        <is>
-          <t>Durante a fiscalização, foi observada a presença de cidadãos que ficaram fiscalizando o serviço conforme o andamento do mesmo. Precisamos mobilizar uma equipe que fiscalize os agentes e os cidadãos em campo.</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="n">
-        <v>12</v>
-      </c>
-      <c r="B12" t="inlineStr">
-        <is>
-          <t>Terminal de Garanhuns (GAR)</t>
-        </is>
-      </c>
-      <c r="C12" t="inlineStr">
-        <is>
-          <t>Durante a fiscalização, foi observada a presença de cidadãos que ficaram fiscalizando o serviço conforme o andamento do mesmo. Precisamos mobilizar uma equipe que fiscalize os agentes e os cidadãos em campo.;Tambem foi observada a presenca de caracteres incompativeis com a resolucao de numero 198392, uma vez que o dispositivo de regulamentacao exige acompanhamento especial durante todo o ciclo; Observa-se tambem lorem ipsumlorem ipsum lorem ipsumlorem ipsumlorem ipsumlorem ipsumlorem ipsumlorem ipsumlorem ipsumlorem ipsumlorem ipsumlorem ipsumlorem ipsumlorem ipsumlorem ipsumlorem ipsum.</t>
-        </is>
-      </c>
-      <c r="D12" t="inlineStr">
-        <is>
-          <t>foto01.jpg;foto02.jpg;foto002.jpg</t>
-        </is>
-      </c>
-      <c r="E12" t="inlineStr">
-        <is>
-          <t>Viga do terminal não posicionada corretamente.;Piso desgastado na entrada do banheiro feminino do TIP em 20/03/2025.;Não conformidade detectada conforme resolucao 12394.</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="n">
-        <v>12</v>
-      </c>
-      <c r="B13" t="inlineStr">
-        <is>
-          <t>Terminal de Caruaru (CAR)</t>
-        </is>
-      </c>
-      <c r="C13" t="inlineStr">
-        <is>
-          <t>Durante a fiscalização, foi observada a presença de cidadãos que ficaram fiscalizando o serviço conforme o andamento do mesmo. Precisamos mobilizar uma equipe que fiscalize os agentes e os cidadãos em campo.;Tambem foi observada a presenca de caracteres incompativeis com a resolucao de numero 198392, uma vez que o dispositivo de regulamentacao exige acompanhamento especial durante todo o ciclo; Observa-se tambem lorem ipsumlorem ipsum lorem ipsumlorem ipsumlorem ipsumlorem ipsumlorem ipsumlorem ipsumlorem ipsumlorem ipsumlorem ipsumlorem ipsumlorem ipsumlorem ipsumlorem ipsumlorem ipsum.</t>
-        </is>
-      </c>
-      <c r="D13" t="inlineStr">
-        <is>
-          <t>foto01.jpg</t>
-        </is>
-      </c>
-      <c r="E13" t="inlineStr">
-        <is>
-          <t>Viga do terminal não posicionada corretamente.</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:E4"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="2" t="inlineStr">
-        <is>
-          <t>ID da Fiscalização</t>
-        </is>
-      </c>
-      <c r="B1" s="2" t="inlineStr">
-        <is>
-          <t>Terminal</t>
-        </is>
-      </c>
-      <c r="C1" s="2" t="inlineStr">
-        <is>
-          <t>Recomendação</t>
-        </is>
-      </c>
-      <c r="D1" s="2" t="inlineStr">
-        <is>
-          <t>Foto</t>
-        </is>
-      </c>
-      <c r="E1" s="2" t="inlineStr">
-        <is>
-          <t>Legenda da Foto</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="n">
-        <v>12</v>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>Terminal de Garanhuns (GAR)</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>Durante a fiscalização, foi observada a presença de cidadãos que ficaram fiscalizando o serviço conforme o andamento do mesmo. Precisamos mobilizar uma equipe que fiscalize os agentes e os cidadãos em campo.</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>foto01.jpg;foto02.jpg</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>Viga do terminal não posicionada corretamente.;Piso desgastado na entrada do banheiro feminino do TIP em 20/03/2025.;</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="n">
-        <v>12</v>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>Terminal de Arcoverde (ARC)</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>Durante a fiscalização, foi observada a presença de cidadãos que ficaram fiscalizando o serviço conforme o andamento do mesmo. Precisamos mobilizar uma equipe que fiscalize os agentes e os cidadãos em campo.</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="n">
-        <v>12</v>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>Terminal do Recife (TIP)</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>Durante a fiscalização, foi observada a presença de cidadãos que ficaram fiscalizando o serviço conforme o andamento do mesmo. Precisamos mobilizar uma equipe que fiscalize os agentes e os cidadãos em campo.;Tambem foi observada a presenca de caracteres incompativeis com a resolucao de numero 198392, uma vez que o dispositivo de regulamentacao exige acompanhamento especial durante todo o ciclo; Observa-se tambem lorem ipsumlorem ipsum lorem ipsumlorem ipsumlorem ipsumlorem ipsumlorem ipsumlorem ipsumlorem ipsumlorem ipsumlorem ipsumlorem ipsumlorem ipsumlorem ipsumlorem ipsumlorem ipsum.</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>foto01.jpg;foto02.jpg;foto01.jpg</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>Viga do terminal não posicionada corretamente.;Piso desgastado na entrada do banheiro feminino do TIP em 20/03/2025.;Lorem ipsum Lorem ipsumLorem ipsumLorem ipsumLorem ipsumLorem ipsumLorem ipsumLorem ipsumLorem ipsumLorem ipsumLorem ipsumLorem ipsumLorem ipsumLorem ipsumLorem ipsumLorem ipsum</t>
+      <c r="C94" t="inlineStr">
+        <is>
+          <t>GAR_2025_07;GAR_2025_09</t>
+        </is>
+      </c>
+      <c r="D94" t="inlineStr">
+        <is>
+          <t>Vigas da testeira necessitando de manutenção estrutural no pátio de manobras do Terminal de Garanhuns, conforme evidenciado nas Fotos 11 e 12.;Viga deteriorada na fachada lateral com armadura de ferro exposta no pátio de manobras do Terminal de Garanhuns, conforme evidenciado nas Fotos 13 e 14.</t>
+        </is>
+      </c>
+      <c r="H94" t="inlineStr">
+        <is>
+          <t>LOREM IPSUM;LOREM IPSUM</t>
+        </is>
+      </c>
+      <c r="I94" t="inlineStr">
+        <is>
+          <t>LOREM IPSUM;LOREM IPSUM</t>
+        </is>
+      </c>
+      <c r="J94" t="inlineStr">
+        <is>
+          <t>LOREM IPSUM;LOREM IPSUM</t>
+        </is>
+      </c>
+      <c r="K94" t="inlineStr">
+        <is>
+          <t>Vigas da testeira necessitando de manutenção estrutural no Terminal de Garanhuns em 22/09/2025;Vigas da testeira necessitando de manutenção estrutural no Terminal de Garanhuns em 22/09/2025.;Viga com armadura de ferro exposta no Terminal de Garanhuns em 22/09/2025;Viga com armadura de ferro exposta no Terminal de Garanhuns em 22/09/2025.</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="n">
+        <v>17</v>
+      </c>
+      <c r="B95" t="inlineStr">
+        <is>
+          <t>Terminal de Petrolina (PET)</t>
+        </is>
+      </c>
+      <c r="C95" t="inlineStr">
+        <is>
+          <t>PET_2025_01;PET_2025_06</t>
+        </is>
+      </c>
+      <c r="D95" t="inlineStr">
+        <is>
+          <t>Fachada necessitando de manutenção e limpeza na entrada do Terminal de Petrolina, conforme evidenciado nas Fotos 15 e 16.;Falta de Limpeza dos vidros do Terminal de Petrolina, conforme evidenciado nas Fotos 17 e 18.</t>
+        </is>
+      </c>
+      <c r="H95" t="inlineStr">
+        <is>
+          <t>LOREM IPSUM;LOREM IPSUM</t>
+        </is>
+      </c>
+      <c r="I95" t="inlineStr">
+        <is>
+          <t>LOREM IPSUM</t>
+        </is>
+      </c>
+      <c r="J95" t="inlineStr">
+        <is>
+          <t>LOREM IPSUM;LOREM IPSUM</t>
+        </is>
+      </c>
+      <c r="K95" t="inlineStr">
+        <is>
+          <t>Fachada necessitando de manutenção e limpeza no Terminal de Petrolina em 24/09/2025.;Fachada necessitando de manutenção e limpeza no Terminal de Petrolina em 24/09/2025.;Vidros necessitando de limpeza no Terminal de Petrolina em 24/09/2025.;Vidros necessitando de limpeza no Terminal de Petrolina em 24/09/2025.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: Mudança nos textos das seções
</commit_message>
<xml_diff>
--- a/src/planilha_fiscalizacao.xlsx
+++ b/src/planilha_fiscalizacao.xlsx
@@ -529,7 +529,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>08/06/2025</t>
+          <t>06/08/2025</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -582,7 +582,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>09/06/2025</t>
+          <t>06/09/2025</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -635,7 +635,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>10/06/2025</t>
+          <t>06/10/2025</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -688,7 +688,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>11/06/2025</t>
+          <t>06/11/2025</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -741,7 +741,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>12/06/2025</t>
+          <t>06/12/2025</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -794,7 +794,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>12/06/2025</t>
+          <t>06/12/2025</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -847,7 +847,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>12/06/2025</t>
+          <t>06/12/2025</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -900,7 +900,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>12/06/2025</t>
+          <t>06/12/2025</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -953,7 +953,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>12/06/2025</t>
+          <t>06/12/2025</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -1006,7 +1006,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>12/06/2025</t>
+          <t>06/12/2025</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -1059,7 +1059,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>12/06/2025</t>
+          <t>06/12/2025</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -1112,7 +1112,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>12/06/2025</t>
+          <t>06/12/2025</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">

</xml_diff>

<commit_message>
feat: Ajuste na formatação das seções e retirada de comentários
</commit_message>
<xml_diff>
--- a/src/planilha_fiscalizacao.xlsx
+++ b/src/planilha_fiscalizacao.xlsx
@@ -529,7 +529,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>06/08/2025</t>
+          <t>08/06/2025</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -582,7 +582,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>06/09/2025</t>
+          <t>09/06/2025</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -635,7 +635,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>06/10/2025</t>
+          <t>10/06/2025</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -688,7 +688,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>06/11/2025</t>
+          <t>11/06/2025</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -741,7 +741,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>06/12/2025</t>
+          <t>12/06/2025</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -794,7 +794,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>06/12/2025</t>
+          <t>12/06/2025</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -847,7 +847,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>06/12/2025</t>
+          <t>12/06/2025</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -900,7 +900,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>06/12/2025</t>
+          <t>12/06/2025</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -953,7 +953,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>06/12/2025</t>
+          <t>12/06/2025</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -1006,7 +1006,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>06/12/2025</t>
+          <t>12/06/2025</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -1059,7 +1059,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>06/12/2025</t>
+          <t>12/06/2025</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -1112,7 +1112,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>06/12/2025</t>
+          <t>12/06/2025</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">

</xml_diff>

<commit_message>
feat: Modificando capa do relatório
</commit_message>
<xml_diff>
--- a/src/planilha_fiscalizacao.xlsx
+++ b/src/planilha_fiscalizacao.xlsx
@@ -529,7 +529,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>08/06/2025</t>
+          <t>06/08/2025</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -582,7 +582,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>09/06/2025</t>
+          <t>06/09/2025</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -635,7 +635,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>10/06/2025</t>
+          <t>06/10/2025</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -688,7 +688,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>11/06/2025</t>
+          <t>06/11/2025</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -741,7 +741,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>12/06/2025</t>
+          <t>06/12/2025</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -794,7 +794,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>12/06/2025</t>
+          <t>06/12/2025</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -847,7 +847,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>12/06/2025</t>
+          <t>06/12/2025</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -900,7 +900,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>12/06/2025</t>
+          <t>06/12/2025</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -953,7 +953,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>12/06/2025</t>
+          <t>06/12/2025</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -1006,7 +1006,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>12/06/2025</t>
+          <t>06/12/2025</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -1059,7 +1059,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>12/06/2025</t>
+          <t>06/12/2025</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -1112,7 +1112,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>12/06/2025</t>
+          <t>06/12/2025</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">

</xml_diff>

<commit_message>
feat(report): Ajusta formatação da tabela de abreviaturas e corrige Key Error
</commit_message>
<xml_diff>
--- a/src/planilha_fiscalizacao.xlsx
+++ b/src/planilha_fiscalizacao.xlsx
@@ -3,11 +3,12 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-21180" yWindow="1785" windowWidth="18900" windowHeight="11385" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fiscalizações" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Não-conformidades " sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Abreviaturas" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="0" fullCalcOnLoad="1"/>
@@ -17,11 +18,28 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="3">
+  <fonts count="6">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <color rgb="FF000000"/>
       <sz val="11"/>
       <scheme val="minor"/>
     </font>
@@ -42,12 +60,27 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="3">
+  <borders count="4">
     <border>
       <left/>
       <right/>
       <top/>
       <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
       <diagonal/>
     </border>
     <border>
@@ -75,12 +108,24 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top"/>
     </xf>
   </cellXfs>
@@ -465,57 +510,57 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="2" t="inlineStr">
+      <c r="A1" s="6" t="inlineStr">
         <is>
           <t>ID da Fiscalização</t>
         </is>
       </c>
-      <c r="B1" s="2" t="inlineStr">
+      <c r="B1" s="6" t="inlineStr">
         <is>
           <t>Data</t>
         </is>
       </c>
-      <c r="C1" s="2" t="inlineStr">
+      <c r="C1" s="6" t="inlineStr">
         <is>
           <t>Hora</t>
         </is>
       </c>
-      <c r="D1" s="2" t="inlineStr">
+      <c r="D1" s="6" t="inlineStr">
         <is>
           <t>Cidade</t>
         </is>
       </c>
-      <c r="E1" s="2" t="inlineStr">
+      <c r="E1" s="6" t="inlineStr">
         <is>
           <t>Local</t>
         </is>
       </c>
-      <c r="F1" s="2" t="inlineStr">
+      <c r="F1" s="6" t="inlineStr">
         <is>
           <t>Pessoal Responsável</t>
         </is>
       </c>
-      <c r="G1" s="2" t="inlineStr">
+      <c r="G1" s="6" t="inlineStr">
         <is>
           <t>Coordenador</t>
         </is>
       </c>
-      <c r="H1" s="2" t="inlineStr">
+      <c r="H1" s="6" t="inlineStr">
         <is>
           <t>Contrato</t>
         </is>
       </c>
-      <c r="I1" s="2" t="inlineStr">
+      <c r="I1" s="6" t="inlineStr">
         <is>
           <t>Período</t>
         </is>
       </c>
-      <c r="J1" s="2" t="inlineStr">
+      <c r="J1" s="6" t="inlineStr">
         <is>
           <t>Assinatura</t>
         </is>
       </c>
-      <c r="K1" s="2" t="inlineStr">
+      <c r="K1" s="6" t="inlineStr">
         <is>
           <t>Relatório Gerado</t>
         </is>
@@ -646,12 +691,12 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="2" t="inlineStr">
+      <c r="A1" s="6" t="inlineStr">
         <is>
           <t>ID da Fiscalização</t>
         </is>
       </c>
-      <c r="B1" s="2" t="inlineStr">
+      <c r="B1" s="6" t="inlineStr">
         <is>
           <t>Legenda da Foto</t>
         </is>
@@ -671,4 +716,131 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C7"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="20" customWidth="1" min="1" max="1"/>
+    <col width="7" customWidth="1" style="4" min="2" max="2"/>
+    <col width="49" customWidth="1" style="4" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>ID da Fiscalização</t>
+        </is>
+      </c>
+      <c r="B1" s="3" t="inlineStr">
+        <is>
+          <t>Sigla</t>
+        </is>
+      </c>
+      <c r="C1" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Definição </t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="30" customHeight="1">
+      <c r="A2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>CAR</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>Terminal Rodoviário de Passageiros de Caruaru</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="30" customHeight="1">
+      <c r="A3" t="n">
+        <v>1</v>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>GAR</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>Terminal Rodoviário de Passageiros de Garanhuns</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>1</v>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>NC</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>Não Conformidade</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>1</v>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>PCD</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>Pessoa com Deficiência</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="30" customHeight="1">
+      <c r="A6" t="n">
+        <v>1</v>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>PET</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>Terminal Rodoviário de Passageiros do Recife</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="n">
+        <v>1</v>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>TRP</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>Terminal Rodoviário de Passageiros</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.511811024" right="0.511811024" top="0.787401575" bottom="0.787401575" header="0.31496062" footer="0.31496062"/>
+  <pageSetup orientation="portrait" paperSize="9"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
feat: Ajusta layout da Capa e implementa controle fino de espaçament
</commit_message>
<xml_diff>
--- a/src/planilha_fiscalizacao.xlsx
+++ b/src/planilha_fiscalizacao.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-21180" yWindow="1785" windowWidth="18900" windowHeight="11385" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fiscalizações" sheetId="1" state="visible" r:id="rId1"/>
@@ -493,20 +493,19 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K3"/>
+  <dimension ref="A1:J3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
     <col width="12" customWidth="1" min="2" max="2"/>
-    <col width="10" customWidth="1" min="3" max="3"/>
-    <col width="21" customWidth="1" min="4" max="4"/>
-    <col width="37" customWidth="1" min="5" max="5"/>
-    <col width="31" customWidth="1" min="6" max="6"/>
+    <col width="13" customWidth="1" min="3" max="3"/>
+    <col width="27" customWidth="1" min="4" max="4"/>
+    <col width="31" customWidth="1" min="5" max="5"/>
+    <col width="34" customWidth="1" min="6" max="6"/>
     <col width="37" customWidth="1" min="7" max="7"/>
-    <col width="17" customWidth="1" min="8" max="8"/>
-    <col width="25" customWidth="1" min="9" max="9"/>
-    <col width="30" customWidth="1" min="10" max="10"/>
-    <col width="18" customWidth="1" min="11" max="11"/>
+    <col width="25" customWidth="1" min="8" max="8"/>
+    <col width="88" customWidth="1" min="9" max="9"/>
+    <col width="18" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -522,22 +521,22 @@
       </c>
       <c r="C1" s="6" t="inlineStr">
         <is>
-          <t>Hora</t>
+          <t>Nº Processo</t>
         </is>
       </c>
       <c r="D1" s="6" t="inlineStr">
         <is>
-          <t>Cidade</t>
+          <t>Nº SEI</t>
         </is>
       </c>
       <c r="E1" s="6" t="inlineStr">
         <is>
-          <t>Local</t>
+          <t>Pessoal Responsável</t>
         </is>
       </c>
       <c r="F1" s="6" t="inlineStr">
         <is>
-          <t>Pessoal Responsável</t>
+          <t>Matrícula do Pessoal Responsável</t>
         </is>
       </c>
       <c r="G1" s="6" t="inlineStr">
@@ -547,20 +546,15 @@
       </c>
       <c r="H1" s="6" t="inlineStr">
         <is>
-          <t>Contrato</t>
+          <t>Período da Fiscalização</t>
         </is>
       </c>
       <c r="I1" s="6" t="inlineStr">
         <is>
-          <t>Período</t>
+          <t>Terminais</t>
         </is>
       </c>
       <c r="J1" s="6" t="inlineStr">
-        <is>
-          <t>Assinatura</t>
-        </is>
-      </c>
-      <c r="K1" s="6" t="inlineStr">
         <is>
           <t>Relatório Gerado</t>
         </is>
@@ -572,27 +566,27 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>06/08/2025</t>
+          <t>12/11/2025</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>10:00:06</t>
+          <t>01/2025</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Joao Recife Pessoas</t>
+          <t>0030200020.007610/2025-19</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Terminal Rodoviário do Recife - TIP</t>
+          <t>Alcides Vieira; Enildo Manoel</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>Alcides Vieira, Enildo Manoel</t>
+          <t>40672015/01</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
@@ -602,20 +596,15 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>Nº 1.041.080/14</t>
+          <t>26/04/2025 a 01/05/2031</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>26/04/2025 a 01/05/2031</t>
-        </is>
-      </c>
-      <c r="J2" t="inlineStr">
-        <is>
-          <t>Alcides Vieira;Enildo Manoel</t>
-        </is>
-      </c>
-      <c r="K2" t="b">
+          <t>Terminal de Recife; Terminal de Caruaru</t>
+        </is>
+      </c>
+      <c r="J2" t="b">
         <v>1</v>
       </c>
     </row>
@@ -625,27 +614,27 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>06/09/2025</t>
+          <t>12/11/2025</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>10:00:07</t>
+          <t>04/2025</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Joao Recife Pessoas</t>
+          <t>0030200020.007610/2025-19</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Terminal Rodoviário do Recife - TIP</t>
+          <t>Alcides Vieira; Enildo Manoel</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Alcides Vieira, Enildo Manoel</t>
+          <t>40672015/01;1796500/02</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
@@ -655,20 +644,15 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>Nº 1.041.080/15</t>
+          <t>26/04/2025 a 01/05/2032</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>26/04/2025 a 01/05/2032</t>
-        </is>
-      </c>
-      <c r="J3" t="inlineStr">
-        <is>
-          <t>Alcides Vieira;Enildo Manoel</t>
-        </is>
-      </c>
-      <c r="K3" t="b">
+          <t xml:space="preserve">Terminal de Recife; Terminal de Caruaru; Terminal de Petrolina; Terminal de Garanhuns </t>
+        </is>
+      </c>
+      <c r="J3" t="b">
         <v>1</v>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: Alteração nos dados da capa
</commit_message>
<xml_diff>
--- a/src/planilha_fiscalizacao.xlsx
+++ b/src/planilha_fiscalizacao.xlsx
@@ -566,7 +566,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>12/11/2025</t>
+          <t>11/12/2025</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -614,7 +614,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>12/11/2025</t>
+          <t>11/12/2025</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">

</xml_diff>

<commit_message>
feat: Adicionando lógica de dados entre a planilha de fiscalização e de dados
</commit_message>
<xml_diff>
--- a/src/planilha_fiscalizacao.xlsx
+++ b/src/planilha_fiscalizacao.xlsx
@@ -18,7 +18,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="6">
+  <fonts count="7">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -49,6 +49,11 @@
       <sz val="11"/>
     </font>
     <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <sz val="11"/>
+    </font>
+    <font>
       <b val="1"/>
     </font>
   </fonts>
@@ -60,12 +65,27 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="4">
+  <borders count="5">
     <border>
       <left/>
       <right/>
       <top/>
       <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
       <diagonal/>
     </border>
     <border>
@@ -108,7 +128,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top"/>
@@ -126,6 +146,9 @@
       <alignment horizontal="center" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top"/>
     </xf>
   </cellXfs>
@@ -509,52 +532,52 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="6" t="inlineStr">
+      <c r="A1" s="7" t="inlineStr">
         <is>
           <t>ID da Fiscalização</t>
         </is>
       </c>
-      <c r="B1" s="6" t="inlineStr">
+      <c r="B1" s="7" t="inlineStr">
         <is>
           <t>Data</t>
         </is>
       </c>
-      <c r="C1" s="6" t="inlineStr">
+      <c r="C1" s="7" t="inlineStr">
         <is>
           <t>Nº Processo</t>
         </is>
       </c>
-      <c r="D1" s="6" t="inlineStr">
+      <c r="D1" s="7" t="inlineStr">
         <is>
           <t>Nº SEI</t>
         </is>
       </c>
-      <c r="E1" s="6" t="inlineStr">
+      <c r="E1" s="7" t="inlineStr">
         <is>
           <t>Pessoal Responsável</t>
         </is>
       </c>
-      <c r="F1" s="6" t="inlineStr">
+      <c r="F1" s="7" t="inlineStr">
         <is>
           <t>Matrícula do Pessoal Responsável</t>
         </is>
       </c>
-      <c r="G1" s="6" t="inlineStr">
+      <c r="G1" s="7" t="inlineStr">
         <is>
           <t>Coordenador</t>
         </is>
       </c>
-      <c r="H1" s="6" t="inlineStr">
+      <c r="H1" s="7" t="inlineStr">
         <is>
           <t>Período da Fiscalização</t>
         </is>
       </c>
-      <c r="I1" s="6" t="inlineStr">
+      <c r="I1" s="7" t="inlineStr">
         <is>
           <t>Terminais</t>
         </is>
       </c>
-      <c r="J1" s="6" t="inlineStr">
+      <c r="J1" s="7" t="inlineStr">
         <is>
           <t>Relatório Gerado</t>
         </is>
@@ -675,12 +698,12 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="6" t="inlineStr">
+      <c r="A1" s="5" t="inlineStr">
         <is>
           <t>ID da Fiscalização</t>
         </is>
       </c>
-      <c r="B1" s="6" t="inlineStr">
+      <c r="B1" s="5" t="inlineStr">
         <is>
           <t>Legenda da Foto</t>
         </is>

</xml_diff>

<commit_message>
feat: Atualizando lógica das legendas de foto e do quadro de fiscalização
</commit_message>
<xml_diff>
--- a/src/planilha_fiscalizacao.xlsx
+++ b/src/planilha_fiscalizacao.xlsx
@@ -128,7 +128,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top"/>
@@ -146,6 +146,9 @@
       <alignment horizontal="center" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -532,52 +535,52 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="7" t="inlineStr">
+      <c r="A1" s="8" t="inlineStr">
         <is>
           <t>ID da Fiscalização</t>
         </is>
       </c>
-      <c r="B1" s="7" t="inlineStr">
+      <c r="B1" s="8" t="inlineStr">
         <is>
           <t>Data</t>
         </is>
       </c>
-      <c r="C1" s="7" t="inlineStr">
+      <c r="C1" s="8" t="inlineStr">
         <is>
           <t>Nº Processo</t>
         </is>
       </c>
-      <c r="D1" s="7" t="inlineStr">
+      <c r="D1" s="8" t="inlineStr">
         <is>
           <t>Nº SEI</t>
         </is>
       </c>
-      <c r="E1" s="7" t="inlineStr">
+      <c r="E1" s="8" t="inlineStr">
         <is>
           <t>Pessoal Responsável</t>
         </is>
       </c>
-      <c r="F1" s="7" t="inlineStr">
+      <c r="F1" s="8" t="inlineStr">
         <is>
           <t>Matrícula do Pessoal Responsável</t>
         </is>
       </c>
-      <c r="G1" s="7" t="inlineStr">
+      <c r="G1" s="8" t="inlineStr">
         <is>
           <t>Coordenador</t>
         </is>
       </c>
-      <c r="H1" s="7" t="inlineStr">
+      <c r="H1" s="8" t="inlineStr">
         <is>
           <t>Período da Fiscalização</t>
         </is>
       </c>
-      <c r="I1" s="7" t="inlineStr">
+      <c r="I1" s="8" t="inlineStr">
         <is>
           <t>Terminais</t>
         </is>
       </c>
-      <c r="J1" s="7" t="inlineStr">
+      <c r="J1" s="8" t="inlineStr">
         <is>
           <t>Relatório Gerado</t>
         </is>
@@ -589,7 +592,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>11/12/2025</t>
+          <t>12/11/2025</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -637,7 +640,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>11/12/2025</t>
+          <t>12/11/2025</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -703,7 +706,7 @@
           <t>ID da Fiscalização</t>
         </is>
       </c>
-      <c r="B1" s="5" t="inlineStr">
+      <c r="B1" s="7" t="inlineStr">
         <is>
           <t>Legenda da Foto</t>
         </is>

</xml_diff>

<commit_message>
feat: Adicionei nova estrutura de paragrafos nas seções
</commit_message>
<xml_diff>
--- a/src/planilha_fiscalizacao.xlsx
+++ b/src/planilha_fiscalizacao.xlsx
@@ -145,10 +145,10 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -592,7 +592,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>12/11/2025</t>
+          <t>11/12/2025</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -640,7 +640,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>12/11/2025</t>
+          <t>11/12/2025</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -706,7 +706,7 @@
           <t>ID da Fiscalização</t>
         </is>
       </c>
-      <c r="B1" s="7" t="inlineStr">
+      <c r="B1" s="6" t="inlineStr">
         <is>
           <t>Legenda da Foto</t>
         </is>

</xml_diff>

<commit_message>
feat: Atualizando formatação da seção de abreviaturas
</commit_message>
<xml_diff>
--- a/src/planilha_fiscalizacao.xlsx
+++ b/src/planilha_fiscalizacao.xlsx
@@ -592,7 +592,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>11/12/2025</t>
+          <t>12/11/2025</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -640,7 +640,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>11/12/2025</t>
+          <t>12/11/2025</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">

</xml_diff>